<commit_message>
feat(sim): assumptions read from the program
assumptions read from the program: start gauges, hit on a sleeping
target, who can be picked, piercing, Double and Triple Attack, stun,
ailment recovery, enemy chant stat, the magic attack chain, effects 71
and 136, dolls, revive items

Fourteen of the sixteen assumptions of sim_setup.xlsx are now readings
with their addresses; one is partly read (the geometry of enemy
formations for piercing) and two are choices of the model (gear and
level of a checkpoint).
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -515,6 +515,7 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,6 +549,11 @@
           <t>Handling</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>What the program says</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -572,12 +578,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Effect 71 adds its value to the "other" bonus once for every status of the target whose class answers yes at slot 0x88 (the buffs and debuffs); effect 136 adds value * the number of the hit record of the action (0x44c60e - 0x44c6b6)</t>
         </is>
       </c>
     </row>
@@ -604,12 +615,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>A plain attack with no multi-hit effect: Triple Attack rolls and adds 3 hits, then Double Attack rolls on its own and adds 2; with neither it hits once: 1, 2, 3 or 5 hits (0x418045 - 0x4180e3)</t>
         </is>
       </c>
     </row>
@@ -636,12 +652,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>The candidates of every pick are the units numbered below 2000 (0x43e6d0). A doll is numbered 2000 + n (0x43a205), a guest ally or a summon 3000 (0x4497ce): none of them can be picked</t>
         </is>
       </c>
     </row>
@@ -668,12 +689,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Spiritual Fantasia (212) is the modifier of attack C of a spell: attack C = attack B * (1 + 212) * (1 + element boost). Waltz (195), effect 335 and the Power of a joint skill multiply the power of the spell only (0x44dcc0 - 0x44e070)</t>
         </is>
       </c>
     </row>
@@ -700,12 +726,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>A party member or an enemy starts at a gauge of (a number below 500, plus 1) / 1000, a guest ally or a summon at the value of a plain action; one battle in five (a roll below 100 under 20) every gauge is (a number below 93) / 100 (0x449130 - 0x449373). An ambush either way (0x44a3d0, effects 267 and 268) is not played: a fight of the simulator starts even</t>
         </is>
       </c>
     </row>
@@ -732,12 +763,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>read; a range if the code does not give it</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Not needed by any rule played: a summon is never a candidate of a pick (0x43e6d0), so its HP decides nothing in a fight. Where the HP comes from is still not read</t>
         </is>
       </c>
     </row>
@@ -764,12 +800,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>read; a range if the code does not give it</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>A doll is built as a copy of its owner's character (0x4f3290 from 0x4fd867): class, previous class, level, the bonus of each stat, the bonus of the resets and the equipment; then HP 9,999. Its stats are its owner's</t>
         </is>
       </c>
     </row>
@@ -796,12 +837,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Bit 11 of the word at file 0x28 of an enemy attack: chanted with INT; bit 12: with RES (0x449b0d - 0x449b38). The 423 attacks that chant have exactly one of the two</t>
         </is>
       </c>
     </row>
@@ -828,12 +874,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>A sleeping target (slot 0xbc, which is the test of sleep: the slots 0xb0 - 0xc4 test poison, freeze, paralysis, sleep and silence in that order) is hit for certain by a blow and by a spell; Fixed accuracy and a direct accuracy value set the chance to value * 100 (0x44aef3 - 0x44afbb, 0x44da4a - 0x44daac)</t>
         </is>
       </c>
     </row>
@@ -860,12 +911,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>partly read</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>A piercing action adds the units of the list its target keeps at 0x64 - 0x68 (0x43fa64). For the party the list is built from how many stand in front and behind (0x43def0): the overlap of two centred rows, which the model uses. For enemies it comes from their place in the formation (0x43e185, not followed); the model applies the same rule to the order of the formation</t>
         </is>
       </c>
     </row>
@@ -892,12 +948,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Stun ends the chant, song, dance and doll of the target, sets its gauge to 0 and is removed at once: no turn is skipped, the next turn comes after a whole wait (0x4fa185 - 0x4fa2f2)</t>
         </is>
       </c>
     </row>
@@ -956,12 +1017,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>The recovery chance of an ailment starts at the third argument of CreateCommand, the turns figure of the action that caused it (0 for every skill of the player, 0 to 6 for enemy attacks, 5 for the items that cause one) and rises by 10 after each failed check (0x47bc03, 0x48d211)</t>
         </is>
       </c>
     </row>
@@ -988,12 +1054,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read in a guide</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Skills of the classes passed through stay usable after a class change, and when the class changes does not change the stats (atwiki dt2-2 page 79)</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1123,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>read</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>An item that revives gives int(max HP * the value of the item / 100) HP, at least 1 (0x5101a4 - 0x5101ca): the 10% of the wiki is the value of the item</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1206,118 +1282,78 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ailment_recovery_start</t>
+          <t>party_size</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>Members of a party</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Bigfoot sealbook test, atwiki dt2-2 page 105: ailments end after 1 to 8 checks of five steps</t>
+          <t>game</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>revive_item_share</t>
+          <t>front_size</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.1</v>
+        <v>3</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>A16: HP of a member brought back by an item, share of max HP</t>
+          <t>Members in the front row of a reference party</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 19: "蘇生時の残HP10%"</t>
+          <t>atwiki dt2-2 page 79</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>party_size</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>gear_min_formations</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Members of a party</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>game</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A12: a zone counts for the gear of the way when it has at least this many random formations; a zone of one or two formations is the place of a single strong enemy whose table gives pieces of +75 to +99</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>floor_data zone tables (St07 to St12)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>front_size</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Members in the front row of a reference party</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 79</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>gear_min_formations</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>gear_level_margin</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>5</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>A12: a zone counts for the gear of the way when it has at least this many random formations; a zone of one or two formations is the place of a single strong enemy whose table gives pieces of +75 to +99</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>floor_data zone tables (St07 to St12)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>gear_level_margin</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>A12: a zone counts for the gear of a checkpoint when its strongest random enemy is at most this many levels above the party; the gear never falls from one checkpoint to the next</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>choice</t>
         </is>

</xml_diff>

<commit_message>
feat(sim): consecutive battles, phase 1 checklist tool, unique skills
consecutive battles, phase 1 checklist tool, unique skills before the
action, fixes of extra actions and per-turn damage caps
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -2625,7 +2625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Battle</t>
+          <t>Battle (several joined by + are fought in a row)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>ペギン先生と七体のペギン</t>
+          <t>ペギン先生と七体のペギン / メルヘン・リトル (連戦)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -3388,8 +3388,10 @@
           <t>St08_0010</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n">
-        <v>45</v>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>45+43</t>
+        </is>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -3403,26 +3405,26 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>C24</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>第六章　本当は怖いおとぎ話</t>
+          <t>第七章　光と影</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>メルヘン・リトル</t>
+          <t>アーヴァンク</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>St08_0010</t>
+          <t>St09_0011</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
@@ -3436,7 +3438,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>C24</t>
+          <t>C25</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -3446,12 +3448,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>アーヴァンク</t>
+          <t>武闘家</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>St09_0011</t>
+          <t>St09_0014</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -3469,7 +3471,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>C25</t>
+          <t>C26</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -3479,16 +3481,16 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>武闘家</t>
+          <t>ミシェルとベアトリーチェ</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>St09_0014</t>
+          <t>St09_0015</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -3502,26 +3504,26 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>C26</t>
+          <t>C27</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>第七章　光と影</t>
+          <t>第八章　妖精国</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>ミシェルとベアトリーチェ</t>
+          <t>森ガーディアン×2</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>St09_0015</t>
+          <t>St10_0010</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -3535,7 +3537,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>C27</t>
+          <t>C28</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3545,16 +3547,16 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>森ガーディアン×2</t>
+          <t>マグ・メルの精霊</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>St10_0010</t>
+          <t>St11_0010</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -3568,7 +3570,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>C28</t>
+          <t>C29</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -3578,7 +3580,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>マグ・メルの精霊</t>
+          <t>カリオペー</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -3587,7 +3589,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -3601,7 +3603,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>C29</t>
+          <t>C30</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3611,16 +3613,18 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>カリオペー</t>
+          <t>蛮野の狂戦士 (二連戦)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>St11_0010</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>44</v>
+          <t>St10_0010</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>43+44</t>
+        </is>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
@@ -3634,7 +3638,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>C30</t>
+          <t>C31</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -3644,12 +3648,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>蛮野の狂戦士</t>
+          <t>マンゴーチン、ドリリアン</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>St10_0010</t>
+          <t>St11_0010</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
@@ -3667,26 +3671,26 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>C31</t>
+          <t>C32</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>第八章　妖精国</t>
+          <t>第九章　絶巓の城</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>マンゴーチン、ドリリアン</t>
+          <t>モビーディック</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>St11_0010</t>
+          <t>St12_0010</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F32" s="2" t="n">
         <v>0</v>
@@ -3700,7 +3704,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>C32</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3710,7 +3714,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>モビーディック</t>
+          <t>デスカタフラクト</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -3719,7 +3723,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F33" s="2" t="n">
         <v>0</v>
@@ -3733,7 +3737,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>C33</t>
+          <t>C34</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3743,16 +3747,18 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>デスカタフラクト</t>
+          <t>闇の女王 (魔力供給装置を破壊、2連戦)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>St12_0010</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>42</v>
+          <t>St12_0040</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>42+43</t>
+        </is>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
@@ -3766,22 +3772,22 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>C34</t>
+          <t>C35</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>第九章　絶巓の城</t>
+          <t>第十章　追憶</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>闇の女王</t>
+          <t>スキャナーズ</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>St12_0040</t>
+          <t>St13_0140</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
@@ -3799,7 +3805,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>C35</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3809,12 +3815,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>スキャナーズ</t>
+          <t>魔神フリード</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>St13_0140</t>
+          <t>St13_0150</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
@@ -3832,22 +3838,22 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>C36</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>第十章　追憶</t>
+          <t>第十一章　魔法都市グリューネワース</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>魔神フリード</t>
+          <t>アイアンメイデン</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>St13_0150</t>
+          <t>St14_1010</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
@@ -3865,22 +3871,22 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>C37</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>第十一章　魔法都市グリューネワース</t>
+          <t>第十二章　はじまりの書</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>アイアンメイデン</t>
+          <t>サマエル</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>St14_1010</t>
+          <t>St15_1060</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
@@ -3898,7 +3904,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>C38</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3908,12 +3914,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>サマエル</t>
+          <t>マリクタウス</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>St15_1060</t>
+          <t>St15_1120</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
@@ -3931,7 +3937,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>C39</t>
+          <t>C40</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3941,87 +3947,23 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>マリクタウス</t>
+          <t>デミウルゴス / アティアルコ (連戦)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>St15_1120</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="n">
-        <v>41</v>
+          <t>St15_1150</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>41+42</t>
+        </is>
       </c>
       <c r="F40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356 (order), pages 24 and 190 (name to enemy by level and HP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>C40</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>第十二章　はじまりの書</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>デミウルゴス</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>St15_1150</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356 (order), pages 24 and 190 (name to enemy by level and HP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>C41</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>第十二章　はじまりの書</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>アティアルコ</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>St15_1150</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 356 (order), pages 24 and 190 (name to enemy by level and HP)</t>
         </is>

</xml_diff>

<commit_message>
docs: decisions of decided: party trios and sub-event bonuses ignored
decisions of decided: party trios and sub-event bonuses ignored; the
level of the reference party is a range he chooses from
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>A party member at a checkpoint has the level of the strongest enemy of the battle (an on-level party)</t>
+          <t>The level of the reference party at a checkpoint. Provisional: the level of the strongest enemy of the battle. To be replaced by a range (direct route, full exploration, levels players report) that the user chooses from</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1091,12 +1091,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>open</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>replaced by the arrival level of phase 2</t>
+          <t>decided by the user (BALANCE_PLAN.md section 6, 2026-10-07); no measure gives a verdict on difficulty before</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: effect rules and assumptions of the engine audit
effect rules and assumptions of the engine audit; coverage regenerated
(effects 209/228, assumptions open 11/26)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -736,7 +736,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>A party member or an enemy starts at a gauge of (a number below 500, plus 1) / 1000, a guest ally or a summon at the value of a plain action; one battle in five (a roll below 100 under 20) every gauge is (a number below 93) / 100 (0x449130 - 0x449373). An ambush either way (0x44a3d0, effects 267 and 268) is not played: a fight of the simulator starts even</t>
+          <t>A party member or an enemy starts at a gauge of (a number below 500, plus 1) / 1000, a guest ally or a summon at the value of a plain action. In a random battle the party strikes first on a roll below 100 under 6 + Preemptive Attack Chance * 100, failing that the enemies on 4 + theirs, stopped by Preemptive Attack Evasion of the other side, certain with Absolute Preemptive Attack (0x44a3d0, 0x4491cf - 0x4491e8); with no ambush, one battle in five every gauge is (a number below 93) / 100 (0x449130 - 0x449373)</t>
         </is>
       </c>
     </row>
@@ -916,12 +916,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>read; a range if the code does not give it</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>A piercing action adds the units of the list its target keeps at 0x64 - 0x68 (0x43fa64). For the party the list is built from how many stand in front and behind (0x43def0): the overlap of two centred rows, which the model uses. For enemies it comes from their place in the formation (0x43e185, not followed); the model applies the same rule to the order of the formation</t>
+          <t>A piercing action adds the units of the list its target keeps at 0x64 - 0x68 (0x43fa64). For the party the list is the overlap of two centred rows (0x43def0). For an enemy it holds the units numbered n + 23, n + 24 and n + 25 when it stands in front, n - 25 to n - 23 when behind (0x43e1ad - 0x43e476): the unit right behind and its two diagonals on a grid 24 wide. How the number of an enemy comes from its place in the formation (the .epd screen positions) is not followed; the model applies the party rule</t>
         </is>
       </c>
     </row>
@@ -1134,6 +1134,326 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>An item that revives gives int(max HP * the value of the item / 100) HP, at least 1 (0x5101a4 - 0x5101ca): the 10% of the wiki is the value of the item</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>A17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>A dodge by Flowing Water Stance is answered by a plain attack of the dodger</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>The skill linked to the status of effect 253 (its counter) is an id the extracted files do not hold</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>the status object of 253, slots 0x34 and 0x3c (0x44b149 - 0x44b1ca)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>read; the linked skill when found</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Against a stab blow 253 is one more evasion term; a roll that lands only without it is a dodge and the bearer then performs the skill linked to the status (0x44b10e - 0x44b20f)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Genjimaru stays until the battle ends</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The constructor of a doll is shared (0x4fd840); the life given to Genjimaru was not followed</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0x48b1f0</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>a range: until the end, or the life of a doll (effect 147)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>A20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Shadow Heart's shadow is a copy of its owner that only attacks and stays until the battle ends</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>What the created unit does and how long it stays were not followed</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0x4378e2</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>a range: one attack, or until the end</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>A21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>An anti-magic zone stops a skill of the magic file, a chanted enemy attack and an action with a magic power</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>The program tests a flag of the record (EnemyAttackData +0x40 bit 2 in memory, and +0x50 bit 5 of another table) that the extracted files do not map yet</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0x41a483, 0x41c184, 0x41e04f</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>partly read</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>read; map the flag to the file</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>A22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>After a turn lost to an ailment the next turn comes after the wait of a plain action</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Phase 4 of the turn (0x4392ef) sets the command kind to 7; the order of turns reads AGI, an action factor of 1 and no defend factor for kind 7 (0x449a24, 0x449d87, 0x44a31c): the wait of a plain action. State 16 is not run: no status counts down or ticks on that turn</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>An action aimed at random units hits as many units as it has hits, each picked with equal chances</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>The picker of target code 1 was not followed</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0x43f450, target code 1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>read; a range if the code does not give it</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>A24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>A dispel (effect 74) removes the statuses that the target's own side put on it, songs and dances excepted</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Which statuses the program counts as buffs (the class answer at slot 0x88) was not listed</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0x4226c4</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>A25</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>The TP of a chanted spell is paid when the chant starts and is lost if the chant breaks</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Where the program takes the TP of a chanted command was not found</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>the command of kind 3</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>a range: paid at the start, or at the cast</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>A26</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>A revived unit acts again after a whole wait</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>The revival writes a hit record of kind 2 (0x48199e); the gauge it leaves was not followed</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0x47e500</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>a range: a whole wait, or its gauge of before</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>A27</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Support Shot strikes the first living target of the plain attack it follows</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>The target of the follow-up attack was not followed</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0x424c42 - 0x42548d</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>read</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: the reference party of the GameFAQs guide
the reference party of the GameFAQs guide: roles, skill plans in the
guide's order, play rules

- roles diva, dark lord, papillon, valkyrie, treasure hunter with their
classes, weapons, rows and characters (Yuni, Yae, Lize, Alisia, Souffle;
Mefmera as a second Papillon until Alisia); the earlier roles stay as
fallbacks - a sequential skill plan per role ('Name:target'), as the
guide gives its priorities - play rules per role from the guide (songs
kept up, Power Charge before the nuke, Berserk kept up, guard buffs) -
still missing: items, meals, sealbooks and enchantments; the weakened
Queen is lost at the level of her route
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -2176,7 +2176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2214,527 +2214,1052 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>tank</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>ally_down</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>revive</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>tank</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>status:170</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>tank</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>party_hp_below:0.5</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>heal:0.5</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 133</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>tank</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>attacker</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>enemy_buffed</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>dispel</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>attacker</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>maid</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>ally_down</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>revive</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>maid</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>ally_hp_below:0.5</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>heal:0.5</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>maid</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>ally_tp_below:0.4</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>tp:0.4</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 120</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>maid</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>status:215</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 129: Replenishing Carol</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>maid</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" t="n">
         <v>5</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>healer</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>ally_down</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>revive</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>healer</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>ally_hp_below:0.6</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>heal:0.6</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>healer</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>ally_ailing</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>cure</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>healer</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" t="n">
         <v>4</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>enemy_buffed</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>dispel</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>healer</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>mage</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>enemy_buffed</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>dispel</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>mage</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>shooter</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>dolls</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>no_doll</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>doll</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 131</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>dolls</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: items when a member falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ally_hp_below:0.35</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>heal:0.35</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: First Aid or an item in an emergency</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>status:215</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "upkeeps Heal/Speed song in boss battles"; the heal song first</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>status:217</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the speed song</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.35</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>tp:0.35</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "helps manage the party TP with cook and self sacrifice"</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>items when a member falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>enemy_buffed</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>dispel</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the dispel on Berserker, for boss buffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>status:191</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>status:26</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "once you get berserk you should also upkeep berserk"</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>items when a member falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>items when a member falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>party_hp_below:0.5</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>heal:0.5</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>status:183</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>status:161</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ally_hp_below:0.35</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>heal:0.35</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
         </is>
       </c>
     </row>
@@ -2749,7 +3274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2833,6 +3358,11 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Skill plan</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3276,6 +3806,341 @@
       <c r="M8" s="2" t="inlineStr">
         <is>
           <t>atwiki dt2-2 pages 131, 147</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Maid</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Bard</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Diva</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Megaphone</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Leather Shield</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Yuni; Ist; Conette</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Yuni Diva; the heal song maxed first, song mastery after, few points elsewhere, then the after-battle regeneration and maid mastery; Lightning March kept up on bosses, Cook and Self-Sacrifice for TP</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Replenishing Carol:max; Song Mastery:max; Lightning March:3; Cook:3; Self-Sacrifice:1; Generous Heart:3; Maid Mastery:3; Blissful Chorale:3; Lightning March:max; Generous Heart:max; Maid Mastery:max</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fighter</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Berserker</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Dark Lord</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Hand Axe</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Kite Shield</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Full Helmet</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Plate Mail</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Yae; Grishna; Luco</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Yae Dark Lord, the dispeller; War Cry max, Power Charge max, level 1 of the nukes, Megaton Press 4, Dark Aura max, then Berserk max or the nukes; one-handed axe with a heavy shield</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>War Cry:max; Power Charge:max; Frost Slash:1; Geo Break:1; Raging Smash:1; Megaton Press:4; Aura Eliminate:1; Dark Aura:max; Berserk:max; Frost Slash:max; Megaton Press:max; Geo Break:max; Axe Mastery:max</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Trickster</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Papillon</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ougi</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Leather Shield</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Lizerietta; Mefmera</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Lize Trickster then Papillon (Joker only at the end of the postgame); Mefmera as a second Papillon until Alisia comes, in the front row; Rose Queen as the area attack, Danger Shoot level 1 and High Risk High Return; the unique guns of the guide are left out, a fan of the zone is worn</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Danger Shoot:1; High Risk, High Return:max; Weapon Mastery:max; Rose Queen:max; Checkmate:1; Anti-Dark Aura:1; Fan Mastery:max; Coffee Break:3; Elegant Dancing:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fighter</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Paladin</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Valkyrie</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Lance</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Kite Shield</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Full Helmet</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Plate Mail</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Alisia</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Alisia Valkyrie; level 1 of Daedalus, Cross Slash and the wind thrust, the useful passives (counter bypass), TP regeneration max, War Cry max, the guard buffs; lance with a shield</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Daedalus Attack:1; Cross Slash:1; Gust Thrust:1; Absolute Attack:1; Guts:1; Auto-Refresh:max; War Cry:max; Spell Guard:max; Lance Mastery:max; Daedalus Attack:max; Parry:max; Cover:max; Protect:max; Moon Curtain:max; Material Guard:max</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Scout</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Treasure Hunter</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Dagger|Kukri</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Leather Shield</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Souffle; Monica; Tsurara</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Souffle Assassin then Treasure Hunter; ambush maxed as soon as possible, mostly passives, the dagger build with Pursuit Stab as its core until the best gun of the postgame</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Awareness:max; Pursuit Stab:max; Dagger Mastery:max; Sharp Stab:1; Murder:max; Treasure Hunt:max; Triple Attack:max; Elusiveness:max; Chain Spike:max</t>
         </is>
       </c>
     </row>
@@ -3290,7 +4155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3316,107 +4181,197 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Maid and healer in one</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: the dispeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: close to mandatory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Mefmera as a second Papillon until Alisia comes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fallback while a role of the guide has nobody yet (early chapters)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>tank</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>maid</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>healer</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>attacker</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>the damage of the party</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>mage</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>the damage of the party</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>shooter</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>a member of another line when a role has nobody</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>dolls</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>a member of another line when a role has nobody</t>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>fallback</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: the shared item bag of the guide party, calibrated
the shared item bag of the guide party, calibrated; songs kept up; boss
preparation

- Sheet Kit (the shop items a party carries into a boss fight) and
kit_count, calibrated to 8 on the anchors C07, C18 and the weakened
Queen; a fruit when a member runs dry - A performer with full song or
dance slots keeps them instead of swapping one for another each turn -
The diva plan takes Self Session level 1 early (GameFAQs Class Skill
info - Maid), so heal and speed songs run together - Sheet Preparation:
the resistance a player raises for a boss the guides warn about (full
Queen: earth 100), A29
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -16,7 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkpoints" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GuideLevels" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joins" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kit" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,6 +509,244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>What it does</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bagel Sandwich</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>HP 500 to one member</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sachertorte</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HP 200 to every member</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fairy Apple</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TP 50 to one member</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mui Kuha Medicine</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>revives a member at 10% HP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fumirul Nectar</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cures every ailment</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Resistance index</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Resistance</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>St12_0040</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Queen of Darkness (all the energy feeds left standing)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207: Curse Wind (instant death) and Evil Eye (sure petrification of a row) "need a countermeasure"; page 147: petrification and instant death are only stopped by earth resistance; docs/FORMULAS.md, effect 121 (0x4834b0): the sure petrification fails at an earth resistance of 100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -895,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1883,6 +2123,38 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>A29</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>For a boss the guides say needs a countermeasure, the reference party raises the named resistance to the value that stops it (sheet Preparation); no other boss-specific gear is modelled</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>It is a choice about the player, not a rule of the program: the guides say a countermeasure is needed but not how many pieces a normal player wears</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207 and the boss notes of the guides</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>a choice for the user (it moves difficulty)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1894,7 +2166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2162,6 +2434,26 @@
       <c r="D13" t="inlineStr">
         <is>
           <t>choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>kit_count</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Items of each row of the sheet Kit (times its share) in the bag the reference party shares in a boss fight. Calibrated 2026-10-08 on the anchors (40 runs each): 8 gives C07 42% at level 13 and 68% at 15 (guide 13 - 15), C18 100% at 25 and 27, the weakened Queen 100% at 50; 5 gives C07 25% and 40%</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>calibration</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2924,17 +3216,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the dispel on Berserker, for boss buffs</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
@@ -2949,17 +3241,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>status:191</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the dispel on Berserker, for boss buffs</t>
         </is>
       </c>
     </row>
@@ -2979,12 +3271,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>status:26</t>
+          <t>status:191</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "once you get berserk you should also upkeep berserk"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
         </is>
       </c>
     </row>
@@ -3004,37 +3296,37 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:26</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "once you get berserk you should also upkeep berserk"</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -3045,71 +3337,71 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
         </is>
       </c>
     </row>
@@ -3120,21 +3412,21 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>status:183</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -3145,21 +3437,21 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
@@ -3170,94 +3462,194 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:183</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>6</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>treasure hunter</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
         <v>3</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ally_hp_below:0.35</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>heal:0.35</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>4</v>
+      </c>
+      <c r="C47" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
         </is>
@@ -3867,12 +4259,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Yuni Diva; the heal song maxed first, song mastery after, few points elsewhere, then the after-battle regeneration and maid mastery; Lightning March kept up on bosses, Cook and Self-Sacrifice for TP</t>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Recommended Party and Best in Slot Gear pages: Yuni Diva; the heal song maxed first, song mastery after, few points elsewhere, then the after-battle regeneration and maid mastery; Self Session level 1 as soon as possible (Class Skill info - Maid) so the heal and speed songs are kept up together, Lightning March kept up on bosses, Cook and Self-Sacrifice for TP</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Replenishing Carol:max; Song Mastery:max; Lightning March:3; Cook:3; Self-Sacrifice:1; Generous Heart:3; Maid Mastery:3; Blissful Chorale:3; Lightning March:max; Generous Heart:max; Maid Mastery:max</t>
+          <t>Replenishing Carol:max; Self Session:1; Song Mastery:max; Lightning March:3; Cook:3; Self-Sacrifice:1; Generous Heart:3; Maid Mastery:3; Blissful Chorale:3; Lightning March:max; Generous Heart:max; Maid Mastery:max</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: boss anchors as a generated checklist
boss anchors as a generated checklist (sheet Anchors,
tools/sim_anchors.py): 4 of 6 met

The guide levels of C07 and C18 and the weakened Queen are met; the
Queen at full strength is not (12% at 60).
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -15,10 +15,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composition" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkpoints" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GuideLevels" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joins" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kit" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anchors" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joins" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kit" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,148 +510,198 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item_ID</t>
+          <t>Chapter</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Characters who join in it</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Share</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>What it does</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Bagel Sandwich</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>HP 500 to one member</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Prologue</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Siena; Luco</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Sachertorte</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>HP 200 to every member</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>第一章</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tsurara</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fairy Apple</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TP 50 to one member</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>第二章</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Yuni</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>26</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Mui Kuha Medicine</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>revives a member at 10% HP</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>第三章</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Lizerietta</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Fumirul Nectar</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>cures every ailment</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>第四章</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Irena; Yae; Conette</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>第五章</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Mefmera; Monica; Eltricia</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>第六章</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Souffle; Grishna</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>第七章</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Lilian; Fiora</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>第八章</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ist; Alisia</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>第九章</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Melvy</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 356</t>
         </is>
       </c>
     </row>
@@ -665,74 +716,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Floor</t>
+          <t>Item_ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Battle</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Boss</t>
+          <t>Share</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Resistance index</t>
+          <t>What it does</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Resistance</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>St12_0040</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>41</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Queen of Darkness (all the energy feeds left standing)</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>6</v>
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bagel Sandwich</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>HP 500 to one member</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>earth</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>100</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 207: Curse Wind (instant death) and Evil Eye (sure petrification of a row) "need a countermeasure"; page 147: petrification and instant death are only stopped by earth resistance; docs/FORMULAS.md, effect 121 (0x4834b0): the sure petrification fails at an earth resistance of 100</t>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sachertorte</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HP 200 to every member</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fairy Apple</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TP 50 to one member</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mui Kuha Medicine</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>revives a member at 10% HP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fumirul Nectar</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cures every ailment</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 19 (the items Rinrin-dou sells; the list does not change with the story)</t>
         </is>
       </c>
     </row>
@@ -742,6 +867,88 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Resistance index</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Resistance</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>St12_0040</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Queen of Darkness (all the energy feeds left standing)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207: Curse Wind (instant death) and Evil Eye (sure petrification of a row) "need a countermeasure"; page 147: petrification and instant death are only stopped by earth resistance; docs/FORMULAS.md, effect 121 (0x4834b0): the sure petrification fails at an earth resistance of 100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2194,7 +2401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2482,6 +2689,26 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>calibration</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>anchor_runs</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>40</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Battles played for each row of the sheet Anchors (tools/sim_anchors.py)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>choice</t>
         </is>
       </c>
     </row>
@@ -6292,198 +6519,223 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chapter</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Characters who join in it</t>
+          <t>Checkpoint</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Battles (blank: those of the checkpoint)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Level (blank: reference level)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Lowest win share</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Highest win share</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>What the source says, read as a win share</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Prologue</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Siena; Luco</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>N01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 37 (Wind Tower, boss)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>the easy way is to reach level 15 and change class: a party at 15 wins most</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>第一章</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Tsurara</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>N02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>13</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 37 (Wind Tower, boss)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>a comment won at level 13: a party at 13 can win</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>第二章</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Yuni</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>N03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>27</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Rousset Royal Villa</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>can overwhelm even bard healing under about level 27: a party at 27 wins most</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>第三章</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Lizerietta</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>N04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207 (Queen of Darkness)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>with the three supply devices destroyed the Queen is weakened and the strength of that point is enough: the party at the reference level of the checkpoint wins most</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>第四章</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Irena; Yae; Conette</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>N05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>60</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207 (Queen of Darkness)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>the Queen at full strength needs about level 55 to 60: a party at 60 wins most</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>第五章</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Mefmera; Monica; Eltricia</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>第六章</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Souffle; Grishna</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>第七章</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Lilian; Fiora</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>第八章</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Ist; Alisia</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>第九章</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Melvy</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 356</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>N06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>55</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207 (Queen of Darkness)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>and a party at 55 wins some</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: the check of a change
the check of a change (phase 1 step 4): touched checkpoints, vanilla
against the change, R08/R10 windows

Battles now report the lowest HP share of the party and the damage of
the enemies per action (R10).
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -2401,7 +2401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2707,6 +2707,106 @@
         </is>
       </c>
       <c r="D15" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>check_runs</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Battles played for each checkpoint a change touches, in vanilla and with the change (sim/measures.py check_change)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>check_won_window</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>R08: the win share of a touched checkpoint may move by this much from vanilla</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>choice: about two standard errors of 40 battles near a share of 0.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>check_time_window</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>R08: the mean length of a won fight may move by this share of the vanilla length</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>check_lowest_hp_window</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>R10: the mean lowest HP share of the party during the fight may move by this much</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>check_pressure_window</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>R10: the damage of the enemies per action against the party's max HP may move by this share of vanilla</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>choice</t>
         </is>

</xml_diff>

<commit_message>
data: superbosses at 99 uncrowned (GameFAQs, EXP Grind/Crowning)
superbosses at 99 uncrowned (GameFAQs, EXP Grind/Crowning); A30 settled
for the code; K02 shape test
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>consistency of the form (C's level and weapon are not stated)</t>
+          <t>the shape (each piece helps, the cap is reached by the third); the size per piece is A30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1303,7 +1303,11 @@
           <t>atwiki dt2-2 page 105</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>test_sim_calibration.ChantSpeed</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1556,6 +1560,11 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 207</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>tools/sim_anchors.py N05, N06</t>
         </is>
       </c>
     </row>
@@ -2613,12 +2622,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>the code as read; the test is not written</t>
+          <t>the code as read (the binary comes before the guides; the user left it to judgement on 2026-10-08). The wiki test is kept as a known discrepancy: chants with chant speed UP may be up to a tenth slower in the model than that test measured</t>
         </is>
       </c>
     </row>
@@ -8703,7 +8712,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8789,7 +8797,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8965,7 +8972,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9006,7 +9012,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9227,7 +9232,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9358,7 +9362,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9489,7 +9492,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9530,7 +9532,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9616,7 +9617,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9657,7 +9657,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9698,7 +9697,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9739,7 +9737,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9780,7 +9777,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9821,7 +9817,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9952,7 +9947,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10074,7 +10068,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Casino VIP Area</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10112,7 +10105,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Casino VIP Area</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10150,7 +10142,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Casino VIP Area</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10188,7 +10179,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Casino VIP Area</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10226,7 +10216,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Casino VIP Area</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -10264,7 +10253,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Casino VIP Area</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -10302,7 +10290,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Casino VIP Area</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -10424,7 +10411,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Wandering Brigade</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -10504,7 +10490,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Four Therian Kings</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -10542,7 +10527,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Four Therian Kings</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10580,7 +10564,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Four Therian Kings</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -10618,7 +10601,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Four Therian Kings</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -10656,7 +10638,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms)</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -10694,7 +10675,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms)</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -10732,7 +10712,6 @@
           <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms)</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10812,7 +10791,6 @@
           <t>atwiki dt2-2 page 356 (異章, the order and the names)</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10850,7 +10828,6 @@
           <t>atwiki dt2-2 page 356 (異章, the order and the names)</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -10888,7 +10865,6 @@
           <t>atwiki dt2-2 page 356 (異章, the order and the names)</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10901,7 +10877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10988,6 +10964,581 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P33</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>99</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P34</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>99</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P35</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>99</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>99</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>99</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>99</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>99</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>99</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>99</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P42</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>99</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P43</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>99</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P44</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>99</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P45</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>99</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P46</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>99</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P47</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>99</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P48</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>99</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P49</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>99</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>99</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>P51</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>99</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>P52</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>99</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P53</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>99</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>P54</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>99</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P55</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>99</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>90 - 99, uncrowned</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), EXP Grind/Crowning</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>the main party is at 90 or 99 by the end of the postgame; without the DLC accessories crowning is not recommended ("you will have an easier time just optimizing your setup"); the DLC is ignored</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: forged enchantments on the reference party
forged enchantments on the reference party (A31): slots by upgrade, the
guide's order, fill 0.75 calibrated; anchors 5/6

Sheets EnchantPlan and EnchantSlots (atwiki page 214, GameFAQs Best in
Slot Gear); the blacksmith from the Dragon Palace.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -19,8 +19,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anchors" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joins" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kit" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnchantPlan" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnchantSlots" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1104,41 +1106,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Floor</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Battle</t>
+          <t>Order</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Boss</t>
+          <t>Slot</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Resistance index</t>
+          <t>Enchant_ID</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Resistance</t>
+          <t>Enchant</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Most per member</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Least upgrade of the piece</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -1147,31 +1154,1768 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>St12_0040</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Queen of Darkness (all the energy feeds left standing)</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>earth</t>
+          <t>Physical attack UP</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>atwiki dt2-2 page 207: Curse Wind (instant death) and Evil Eye (sure petrification of a row) "need a countermeasure"; page 147: petrification and instant death are only stopped by earth resistance; docs/FORMULAS.md, effect 121 (0x4834b0): the sure petrification fails at an earth resistance of 100</t>
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>51</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>104</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Physical attack UP</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>104</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>29</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Physical attack UP</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>51</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>104</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>29</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Physical attack UP</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>21</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>51</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>104</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>29</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Physical attack UP</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>51</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>104</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>29</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Physical attack UP</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>21</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>51</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>104</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>29</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Physical attack UP</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>21</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>5</v>
+      </c>
+      <c r="G27" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>51</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>104</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>29</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Physical attack UP</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: weapon "Phys ATK up, Phys accuracy up, Speed up"</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>21</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>10</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>51</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>104</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>37</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Magic attack UP</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>54</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Chant speed UP</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>3</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>21</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" t="n">
+        <v>10</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>51</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>104</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>maid</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>37</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Magic attack UP</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>maid</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>54</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Chant speed UP</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>maid</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>21</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>5</v>
+      </c>
+      <c r="G41" t="n">
+        <v>10</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>maid</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>51</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>maid</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>5</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>104</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>5</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>37</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Magic attack UP</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>54</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Chant speed UP</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>21</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" t="n">
+        <v>10</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>4</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>51</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>104</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>5</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>37</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Magic attack UP</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>54</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Chant speed UP</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>3</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: caster weapon "Mag Power UP, Chant Speed UP"; chant speed caps at three pieces</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>3</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>21</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>AGI UP</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G51" t="n">
+        <v>10</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>51</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Speed UP</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>5</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>104</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Elemental resistance UP</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>5</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear: "always prioritize AGI UP (one per equip piece is max) &gt; Speed UP (up to 5 across all gear) &gt; +15 Elem Resists"; atwiki dt2-2 page 214: ATK to AGI UP need the piece at +10; weapons take no defensive enchantment, armour no offensive one</t>
         </is>
       </c>
     </row>
@@ -1181,6 +2925,158 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Least upgrade</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Slots</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 214: 2 slots up to +49, 3 from +50, 4 from +75</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 214: 2 slots up to +49, 3 from +50, 4 from +75</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 214: 2 slots up to +49, 3 from +50, 4 from +75</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Resistance index</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Resistance</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>St12_0040</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Queen of Darkness (all the energy feeds left standing)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207: Curse Wind (instant death) and Evil Eye (sure petrification of a row) "need a countermeasure"; page 147: petrification and instant death are only stopped by earth resistance; docs/FORMULAS.md, effect 121 (0x4834b0): the sure petrification fails at an earth resistance of 100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1579,7 +3475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2612,7 +4508,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>The chant test of atwiki dt2-2 page 105 (K02) does not fit it: from 0 to 4 pieces of UP the turns of the fast unit were 61, 51, 40, 31, 31 and 35 with two UP and a MiniUP. Those fit a straight line of slope 0.40 per point of bonus (not the 0.51 the form gives when fitted at 0 pieces) and a cap of 0.6; under the code, three UP and two UP plus a MiniUP are both 0.5 and should match</t>
+          <t>The chant test of atwiki dt2-2 page 105 (K02) does not fit it: from 0 to 4 pieces of UP the turns of the fast unit were 61, 51, 40, 31, 31 and 35 with two UP and a MiniUP. Those fit a straight line of slope 0.40 per point of bonus (not the 0.51 the form gives when fitted at 0 pieces) and a cap of 0.6; under the code, three UP and two UP plus a MiniUP are both 0.5 and should match. atwiki page 214 also says the cap of chant speed UP rose to three pieces (+60%) from 2.5 (+50%) in the first game</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2628,6 +4524,38 @@
       <c r="F30" t="inlineStr">
         <is>
           <t>the code as read (the binary comes before the guides; the user left it to judgement on 2026-10-08). The wiki test is kept as a known discrepancy: chants with chant speed UP may be up to a tenth slower in the model than that test measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>The reference party has a share of the enchantment slots of its gear filled by forging (sheet EnchantPlan, setting enchant_fill), from the dungeon of the blacksmith on; no drop enchantments before it and no unique pieces</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>How much a normal player forges is not in any source: the share is calibrated on the anchors</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GameFAQs Best in Slot Gear; atwiki pages 214 and 207</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>a choice the user took on 2026-10-08 (model enchanted gear)</t>
         </is>
       </c>
     </row>
@@ -2642,7 +4570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3050,6 +4978,46 @@
       <c r="D20" t="inlineStr">
         <is>
           <t>choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>enchant_fill</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Share of the enchantment slots of its gear a reference member has filled by forging, in the order of the sheet EnchantPlan (A31). Calibrated 2026-10-08 on the sheet Anchors, 30 battles each: the full Queen at 60 wins 13% with 0, 40% with 0.25, 47% with 0.5, 67% with 0.75, 87% with 1; at 55 she stays at 0 - 17% whatever the share. 0.75 is the least that meets N05; the other anchors do not move</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>calibration</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>forge_from_dungeon</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>First dungeon (the number of its floors, St04 = Dragon Palace) from which the blacksmith can be met and enchantments forged</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 214: first met in the Dragon Palace</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: piercing actions against enemies follow the formation slots
piercing actions against enemies follow the formation slots (A10 read);
random targets (A23) and A29 settled
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -3865,7 +3865,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>A piercing attack hits its target and one unit of the other row</t>
+          <t>A piercing attack hits its target and the units of the other row behind it: for enemies, those whose formation slot is within one of the target's (numbered 1000 + slot in front, 1024 + slot behind); for the party, the overlap of the two rows centred on each other</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3880,12 +3880,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>read; a range if the code does not give it</t>
+          <t>read: 0x439e0e, 0x43e1ad - 0x43e476, 0x43fa64</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>An action aimed at random units hits as many units as it has hits, each picked with equal chances</t>
+          <t>An action aimed at random units makes one pick per hit with equal chances, with repeats; with effect 112 the picks do not repeat and stop when no unit is left</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4294,12 +4294,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>read; a range if the code does not give it</t>
+          <t>read: 0x43f8a2 - 0x43f9a4 and its three callers (argument 5 is effect 112; the enemy caller passes no fixed target)</t>
         </is>
       </c>
     </row>
@@ -4486,12 +4486,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>a choice for the user (it moves difficulty)</t>
+          <t>the user's decision of 2026-10-08 (option 1: the reference party wears prepared, enchanted gear)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: dispel removes the list the program gives (A24 read)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>A dispel (effect 74) removes the statuses that the target's own side put on it, songs and dances excepted</t>
+          <t>A dispel (effect 74), on one roll of its value, removes every status of a fixed list of effects (Battle.dispellable): some always, the stat and power ones while their value is not negative; songs, dances and ailments never</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4326,12 +4326,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>read: 0x4226c4 - 0x422783 (one roll, then every status of the list), 0x4fb1f0, slots 0x64 and 0x54 of the status classes, 0x479df0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: genjimaru lasts 3 turns (A18 read)
genjimaru lasts 3 turns (A18 read); Support Shot (A27) read; A25 and A26
settled as choices
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -4156,7 +4156,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Genjimaru stays until the battle ends</t>
+          <t>Genjimaru stays three turns; it is not ended with the dolls of its owner</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4171,12 +4171,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>a range: until the end, or the life of a doll (effect 147)</t>
+          <t>read: 0x48b319 - 0x48b32c pushes a life of 3 to the doll constructor 0x4fd840, whose second argument a doll skill fills with its effect 147 (0x4843f0 - 0x4844d6)</t>
         </is>
       </c>
     </row>
@@ -4358,12 +4358,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>a range: paid at the start, or at the cast</t>
+          <t>a choice: paid when the chant starts. The payment was traced to the unit's slot 0x11c (0x4fd250, the cost with enchantments 246 - 248) through 0x4f6dd0, which no battle code calls directly; it only matters for a chant broken before its end</t>
         </is>
       </c>
     </row>
@@ -4390,12 +4390,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>a range: a whole wait, or its gauge of before</t>
+          <t>a choice: a whole wait. The revival (0x481997 - 0x4819d8) writes a record of kind 2 with int(max HP * value) and nothing about the gauge; the code that applies the record was not found</t>
         </is>
       </c>
     </row>
@@ -4422,12 +4422,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>read: 0x424c42 - 0x424dc1 (the hit records of the plain attack, each target still standing)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: anti-magic zones stop spells by the flag of the record (A21 read)
anti-magic zones stop spells by the flag of the record (A21 read);
Shadow Heart's shadow lasts 3 turns (A20 read)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -4188,7 +4188,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Shadow Heart's shadow is a copy of its owner that only attacks and stays until the battle ends</t>
+          <t>Shadow Heart's shadow is a copy of its owner that makes plain attacks for three turns; one at a time</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4203,12 +4203,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>a range: one attack, or until the end</t>
+          <t>read: 0x4378e2 - 0x437a44 (roll, one shadow per owner, constructor 0x4fe2e0 with a life of 3 and no actions)</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>An anti-magic zone stops a skill of the magic file, a chanted enemy attack and an action with a magic power</t>
+          <t>An anti-magic zone stops a skill of the magic file and an enemy attack flagged as a spell (bit 2 of the word at file 0x28); techniques and other enemy attacks go through</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4235,12 +4235,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>read; map the flag to the file</t>
+          <t>read: 0x41a483 (+0x40 in memory is the word at file 0x28: its bit 2 is set on 420 of the 423 chanted enemy attacks), 0x41e04f (the spell table 0x738a58), 0x41c184 (table 0x738a54, the joint skills by elimination: techniques are 0x738a64 with enchantment 246, spells 0x738a58 with 248)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: A17 and A28 settled; every assumption of the simulator read or a
A17 and A28 settled; every assumption of the simulator read or a stated
choice (0 of 30 open)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -4134,12 +4134,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>read; the guide where the code is not followed</t>
+          <t>a choice: a plain attack. Read: the status performs the technique at its +0x14 or else the enemy attack at its +0x18 (slots 0x34 and 0x3c, 0x421e89 - 0x421ed0), nothing when both are -1; the effect slots of Knock Down and Pretend carry no id (their tail is 0) and the code that fills the two fields was not found</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4454,12 +4454,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>partly read</t>
+          <t>read in a guide</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>read; the guide where the code is not followed</t>
+          <t>the code for their number, life and action (0x484330); the GameFAQs guide for what ends them (they cannot be interrupted and vanish with the sniper)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: phase 1 closed with one known limit
phase 1 closed with one known limit (N06, full Queen at 55) to confirm;
meals probed and left out (A32)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,6 +557,11 @@
           <t>What the source says, read as a win share</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Known limit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -730,6 +735,11 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>and a party at 55 wins some</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Not met by the model: 0 - 17% at level 55 whatever the share of forged enchantments, and 0 - 7.5% with the best meal of the ice cream and ramen shops in the best case (its buffs at the start of the fight, 40 battles, 2026-10-09). What a player at 55 adds beyond the model (unique pieces, character sealbooks, a party built for this fight) is not modelled. The fight is optional (the three supply devices weaken the Queen, N04, met). Closed as a known limit, for the user to confirm</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4556,6 +4566,38 @@
       <c r="F31" t="inlineStr">
         <is>
           <t>a choice the user took on 2026-10-08 (model enchanted gear)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>A32</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>The reference party eats no meal of the ice cream and ramen shops before a boss</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>The shops are met at random inside a dungeon, after five battles and fifty steps on a floor, and only cheap dishes are offered in low-rank dungeons; the buffs of a dish last 3 to 9 turns (Protect 9, Accelerator 3), and five steps on the map are a turn, so they rarely reach a boss. A probe with the best dish at the start of the full Queen fight (40 battles): 31-Layer Ice Cream (Protect 5, Accelerator 5) 0% at 55, 75% at 60 (60% without); Miracle Shake (Divine Shield 5) 7.5% at 55, 50% at 60</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 pages 194 (the shops and their menus) and 350 (when a shop appears); FoodMenu of vanilla_source_of_truth.xlsx</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>a choice: meals are left out of the preparation for a boss</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: the doll line in the model
the doll line in the model: a Soul Summoner role, two dolls kept with
Double Puppet, slot_share measure

The slot of the first Papillon filled by every line: the Spieler line
sits below the Fighter and Scout lines (Papillon about two thirds of
them, the doll line about one third).
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -5114,7 +5114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>no_doll</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 131</t>
+          <t>atwiki dt2-2 page 131; a free doll slot is filled (two with Double Puppet, page 146)</t>
         </is>
       </c>
     </row>
@@ -6298,6 +6298,56 @@
       <c r="E47" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>doll_slot_free</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>doll</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7179,6 +7229,68 @@
       <c r="N13" t="inlineStr">
         <is>
           <t>Awareness:max; Pursuit Stab:max; Dagger Mastery:max; Sharp Stab:1; Murder:max; Treasure Hunt:max; Triple Attack:max; Elusiveness:max; Chain Spike:max</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Doll Master</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Soul Summoner</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Ougi</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Spartan; Oracles; Catalina; Doll Mastery; Double Puppet; Mercidarian; Musiy; Perdurabo; Destiny Line; Coffee Break; Weapon Mastery</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Lizerietta; Lilian; Mefmera</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 pages 131, 146 (the doll line to its top: Double Puppet keeps two dolls, the strongest dolls of the Soul Summoner); for the doll rows of the register (U02, J18), not in the composition</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: a doll order of preference in the play rules
a doll order of preference in the play rules (GameFAQs: Mercidarian the
best doll); Soul Summoner plan raises it sooner
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -5642,12 +5642,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>doll</t>
+          <t>doll:Spartan|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 131; a free doll slot is filled (two with Double Puppet, page 146)</t>
+          <t>atwiki dt2-2 page 131; a free doll slot is filled (two with Double Puppet, page 146); GameFAQs Class Skill info - Spieler: Spartan first, Oracles "don't bother"</t>
         </is>
       </c>
     </row>
@@ -6317,12 +6317,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>doll</t>
+          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled</t>
+          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
         </is>
       </c>
     </row>
@@ -7280,7 +7280,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Spartan; Oracles; Catalina; Doll Mastery; Double Puppet; Mercidarian; Musiy; Perdurabo; Destiny Line; Coffee Break; Weapon Mastery</t>
+          <t>Spartan; Catalina; Doll Mastery; Double Puppet; Mercidarian; Perdurabo; Musiy; Oracles; Destiny Line; Coffee Break; Weapon Mastery</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 131, 146 (the doll line to its top: Double Puppet keeps two dolls, the strongest dolls of the Soul Summoner); for the doll rows of the register (U02, J18), not in the composition</t>
+          <t>atwiki dt2-2 pages 131, 146 (the doll line to its top: Double Puppet keeps two dolls, the strongest dolls of the Soul Summoner); for the doll rows of the register (U02, J18), not in the composition; GameFAQs faqs/80834, Class Skill info - Spieler: Mercidarian "by far best doll", Double Puppet a must, Oracles "don't bother", Musiy not worth it</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: roles of the six missing advanced classes
roles of the six missing advanced classes; first T05 class measures
recorded (to measure again after the simulator audit)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -5114,7 +5114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6351,6 +6351,581 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>magical princess</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>status:189</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Magical Change kept up (page 137)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>magical princess</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>items when a member falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>party_hp_below:0.5</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>heal:0.5</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>heals when the party is low</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>enemy_buffed</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>dispel</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Dispel against boss buffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>status:168</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Accelerator kept up</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>status:172</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Amplify kept up</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>6</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>status:163</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Sun Veil kept up</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>7</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>kunoichi</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>status:101</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Shadow Clone kept up (page 142)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>kunoichi</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>mistress</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Resurrect or items</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>mistress</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>status:215</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>the heal song kept up</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>mistress</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>status:161</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>War Cry kept up</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>mistress</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>items when a member falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>status:195</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Fascinating Waltz on the enemies</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>status:201</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Dumbing Mazurka on the enemies</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.35</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>tp:0.35</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Cook</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>5</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>joker</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>ally_down</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>revive</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>items when a member falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>joker</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>status:48</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Trump Card on bosses (page 148)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>joker</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>the mean damage per time of every skill</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6362,7 +6937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7291,6 +7866,388 @@
       <c r="M14" t="inlineStr">
         <is>
           <t>atwiki dt2-2 pages 131, 146 (the doll line to its top: Double Puppet keeps two dolls, the strongest dolls of the Soul Summoner); for the doll rows of the register (U02, J18), not in the composition; GameFAQs faqs/80834, Class Skill info - Spieler: Mercidarian "by far best doll", Double Puppet a must, Oracles "don't bother", Musiy not worth it</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>magical princess</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Magic User</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sorceress</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Magical Princess</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Longsword</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Leather Shield</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Fireball; Ice Edge; Fire Blast; Magical Change; Magical Spark; Sword Mastery; Magical Slash; Rainbow Flash; Double Attack; Accelerator; Magic Barrier; Guts; Cover</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Melvy; Siena; Eltricia; Fiora; Irena</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 137 (Magical Change, then her attacks; sword); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Magic User</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Enchantress</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Sage</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Magic Hat</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Robe</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Heal; Circle Brave; Circle Protect; Accelerator; Amplify; Sun Veil; Dispel; Esarhaddon; Slow; Stab Guard; Slash Guard; Bash Guard; Prism Dawn; Fast Cast; Sleep; Silence</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Fiora; Irena; Siena; Melvy; Eltricia</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 138 (support: party buffs, ailments, automatic cure); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>kunoichi</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Scout</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Kunoichi</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Tantou</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Sharp Stab; Sleep Sting; Stun Sting; Dagger Mastery; Shadow Clone; Ninja Piledriver; Katana Mastery; Shadow Sew; Fire Scroll; Water Scroll; Lightning Scroll; Wind Scroll; Earth Scroll; Light Scroll; Barrage; Dual Wield; Phoenix</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Tsurara; Monica; Souffle</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 142 (fast debuffer: Shadow Clone, ninja arts); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mistress</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Maid</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Bard</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mistress</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Whip</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Replenishing Carol; Hard Whipping; Whip Mastery; Enticing Love; Absolute Obedience; War Cry; Song Mastery; Carrot and Stick; Counter Whip; Ecstasy; Knock Down</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Conette; Ist; Yuni</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 144 (sub-attacker who supports with her Bard skills, back row); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Maid</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dancer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Etoile</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Dagger</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Fascinating Waltz; Dance Mastery; Gloomy Tango; Dumbing Mazurka; On Stage; Debilitating Salsa; Emaciating Hopak; Magnificent Steps; Alluring Samba; Gravitating Polka; Cook; Clean</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Ist; Conette; Yuni</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 145 (two dances at once, strong on bosses); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages (Dumbing Mazurka top tier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>joker</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Trickster</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Joker</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Hand Axe</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Leather Shield</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Leather Helmet</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Leather Armor</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>front</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Danger Shoot; High Risk, High Return; Checkmate; Trump Card; Axe Mastery; Weapon Mastery; Mad Zapper; Avenger; Murder; Triple Joker; Life Bringer; Heaven or Hell</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Lizerietta; Mefmera; Lilian</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 148 (buffs and chance skills; Trump Card is her core); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sim): audit findings: passives Elegant Dancing and Adaptation act
audit findings: passives Elegant Dancing and Adaptation act, item cures
read from the exe, boss condition, status rules ignore hit properties,
kunoichi on darts with Dual Wield; sim_audit usage phase

- Elegant Dancing (285) and Adaptation (248) were read only among
statuses; a passive is a status that never ends - item types 6 (cure one
ailment at random, 0x50fb30) and 7 (cure all, 0x50fe20); act_cure uses
items too; a common rule (role '*') cures petrification, freeze,
paralysis and sleep (atwiki p317, Samael) - condition 'boss' was never
true (Trump Card never used): now a fixed battle of the story -
act_status took effect 26 as a hit property (Frost Slash for Berserk):
only kinds 4 and 5 count - off-hand weapon only with Dual Wield;
kunoichi role on Darts + Tantou (atwiki p142) - sage, tank: party buffs
from their pages; sim_audit fights in the reference party, usage phase
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -5114,7 +5114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5154,7 +5154,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>*</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -5162,453 +5162,453 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>ally_ailing:120;114;115;116</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>cure:120;114;115;116</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>atwiki dt2-2 page 317 (VS Samael: cure the petrification of Chaos Eye, items too): any member cures an ailment that takes turns away (petrification, freeze, paralysis, sleep) before its own plan</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>status:170</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>attacker</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the dispel on Berserker, for boss buffs</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:191</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.5</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>status:26</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "once you get berserk you should also upkeep berserk"</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.4</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>tp:0.4</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 129: Replenishing Carol</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: First Aid or an item in an emergency</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "upkeeps Heal/Speed song in boss battles"; the heal song first</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.6</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>heal:0.6</t>
+          <t>status:217</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the speed song</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ally_ailing</t>
+          <t>ally_tp_below:0.35</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>cure</t>
+          <t>tp:0.35</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "helps manage the party TP with cook and self sacrifice"</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>dolls</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>doll:Spartan|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 131; a free doll slot is filled (two with Double Puppet, page 146); GameFAQs Class Skill info - Spieler: Spartan first, Oracles "don't bother"</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>dolls</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>etoile</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>shooter</t>
+          <t>etoile</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -5617,198 +5617,198 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:195</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Fascinating Waltz on the enemies</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>dolls</t>
+          <t>etoile</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>doll_slot_free</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>doll:Spartan|Catalina|Oracles</t>
+          <t>status:201</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 131; a free doll slot is filled (two with Double Puppet, page 146); GameFAQs Class Skill info - Spieler: Spartan first, Oracles "don't bother"</t>
+          <t>Dumbing Mazurka on the enemies</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dolls</t>
+          <t>etoile</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.35</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.35</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Cook</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>etoile</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: First Aid or an item in an emergency</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_hp_below:0.6</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>heal:0.6</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "upkeeps Heal/Speed song in boss battles"; the heal song first</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_ailing</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>status:217</t>
+          <t>cure</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the speed song</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.35</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>tp:0.35</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "helps manage the party TP with cook and self sacrifice"</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -5829,7 +5829,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>dark lord</t>
+          <t>joker</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -5854,7 +5854,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>dark lord</t>
+          <t>joker</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -5862,24 +5862,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>status:48</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>Trump Card on bosses (page 148)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>dark lord</t>
+          <t>joker</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -5887,28 +5887,28 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the dispel on Berserker, for boss buffs</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>dark lord</t>
+          <t>kunoichi</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -5917,23 +5917,23 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>status:191</t>
+          <t>status:101</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
+          <t>Shadow Clone kept up (page 142)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>dark lord</t>
+          <t>kunoichi</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -5942,98 +5942,98 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>status:26</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "once you get berserk you should also upkeep berserk"</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>dark lord</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>status:189</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>Magical Change kept up (page 137)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -6047,14 +6047,14 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -6072,14 +6072,14 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -6087,24 +6087,24 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>ally_hp_below:0.5</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -6112,24 +6112,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_tp_below:0.4</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>tp:0.4</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+          <t>atwiki dt2-2 page 120</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -6142,19 +6142,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>status:183</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+          <t>atwiki dt2-2 page 129: Replenishing Carol</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -6167,173 +6167,173 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
+          <t>Resurrect or items</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+          <t>the heal song kept up</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>War Cry kept up</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>doll_slot_free</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -6347,14 +6347,14 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -6362,24 +6362,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>status:189</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Magical Change kept up (page 137)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -6387,17 +6387,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>heals when the party is low</t>
         </is>
       </c>
     </row>
@@ -6408,21 +6408,21 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>Dispel against boss buffs</t>
         </is>
       </c>
     </row>
@@ -6433,21 +6433,21 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>heals when the party is low</t>
+          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up)</t>
         </is>
       </c>
     </row>
@@ -6458,21 +6458,21 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Dispel against boss buffs</t>
+          <t>atwiki dt2-2 page 138 (Circle Protect kept up)</t>
         </is>
       </c>
     </row>
@@ -6483,7 +6483,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -6492,12 +6492,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>status:168</t>
+          <t>status:163</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Accelerator kept up</t>
+          <t>Sun Veil kept up</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -6542,12 +6542,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>status:163</t>
+          <t>status:168</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Sun Veil kept up</t>
+          <t>Accelerator (one ally, 3 turns) after the party-wide buffs</t>
         </is>
       </c>
     </row>
@@ -6558,7 +6558,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -6579,7 +6579,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>kunoichi</t>
+          <t>shooter</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -6592,98 +6592,98 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>status:101</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Shadow Clone kept up (page 142)</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>kunoichi</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Resurrect or items</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>the heal song kept up</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -6692,73 +6692,73 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>status:170</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>War Cry kept up</t>
+          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 133</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>etoile</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>etoile</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -6767,162 +6767,262 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>status:195</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Fascinating Waltz on the enemies</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>etoile</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>status:201</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Dumbing Mazurka on the enemies</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>etoile</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.35</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>tp:0.35</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Cook</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>etoile</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>joker</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>joker</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>status:48</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Trump Card on bosses (page 148)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>joker</t>
+          <t>valkyrie</t>
         </is>
       </c>
       <c r="B72" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
         <v>3</v>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>party_hp_below:0.5</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>heal:0.5</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>4</v>
+      </c>
+      <c r="C74" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>status:183</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>status:161</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>6</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>the mean damage per time of every skill</t>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
         </is>
       </c>
     </row>
@@ -8021,6 +8121,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>Darts</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>Tantou</t>
         </is>
       </c>
@@ -8046,7 +8151,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Sharp Stab; Sleep Sting; Stun Sting; Dagger Mastery; Shadow Clone; Ninja Piledriver; Katana Mastery; Shadow Sew; Fire Scroll; Water Scroll; Lightning Scroll; Wind Scroll; Earth Scroll; Light Scroll; Barrage; Dual Wield; Phoenix</t>
+          <t>Phoenix; Projectile Mastery; Dual Wield; Shadow Clone; Ninja Piledriver; Fire Scroll; Earth Scroll; Lightning Scroll; Water Scroll; Wind Scroll; Light Scroll; Shadow Sew; Barrage; Evade; Elusiveness; Adaptation</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -8056,7 +8161,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 142 (fast debuffer: Shadow Clone, ninja arts); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
+          <t>atwiki dt2-2 page 142 (fast debuffer: Shadow Clone, ninja arts); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages; atwiki dt2-2 page 142: Phoenix makes a throwing weapon the main weapon, Dual Wield adds the ATK of a second weapon in the left hand (which does not count as the equipped weapon)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sim): imperial Guard kept its negative value
imperial Guard kept its negative value; random-move skills scored by
expected damage; audit readings and checklist

- build_member took max(0, value): Imperial Guard (308, negative) was
always 0 - Roulette, Magic Box, Showtime, Heaven or Hell: the weighted
mean of their results (Joker weights with Triple Joker) - sheet
AuditReadings: 12 of 12 passives seen doing nothing read (11 context,
Soul Seal a model gap: no sealbook) - sim_audit passives in four slices,
one process each
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnchantSlots" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditReadings" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3479,6 +3480,292 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>247 Katana Mastery</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>It raises the ATK and RES of a katana in the main hand. No role holds one there: the attacker fights with a Claymore, and the Kunoichi holds her Tantou in the left hand, which a mastery ignores (atwiki dt2-2 page 142).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>253 Heal Mastery</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>At C18 the Sage never heals (the party stays above half HP under the songs of the Diva). It acts at P24 (recheck 2026-10-09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>255 Mini Auto-Recovery</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>At C18 the songs of the Diva keep every member at full HP. It acts at C34 and P24 (recheck 2026-10-09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>264 Knock Down</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>It answers long-range physical blows with a weapon; Samael (C38) has none against the Mistress. It acts at P24 (recheck 2026-10-09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>269 Murder</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Instant death on a critical blow: every boss tried (C18, C34, P24) is immune to instant death. It is a rule for common enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>272 Preparation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Speed below 40% HP: at C18 the attacker never falls that low. It acts at C34 and P24 (recheck 2026-10-09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>275 Anti-Dark Aura</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>No Dark Aura in the C18 fight. It acts at C34 (recheck 2026-10-09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>281 Concentrate</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Only a physical hit can break a chant (docs/FORMULAS.md 2.5, 0x44d1f3). The mage stands in the back row: three such hits in three C34 fights, each too small to break a chant with or without it; none at P24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>285 Caution</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>It rolls against an ambush, and only random battles start with one (Battle.ambush): the audit plays boss fights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>286 Awareness</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>It raises the chance of a first strike, and only random battles have one (Battle.ambush): the audit plays boss fights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>297 Soul Seal</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>model gap</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>It adds the stats of the enemy of her sealbook to her dolls; the reference parties carry no sealbook yet (BALANCE_PLAN, sealbooks stay in the model; theme T10). Until then the Soul Summoner is measured without it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>307 Triple Joker</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>It changes the weights of the random skills of the Joker; at C38 her other skills score higher and she draws none. It acts at C34 (recheck 2026-10-09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>277 Imperial Guard</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>It never acted: build_member kept max(0, value) and its values are negative. Fixed 2026-10-09 (the larger figure by size); it acts at C38.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>306 Elegant Dancing</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Read only among statuses; a passive is a status that never ends (FORMULAS 12.15). Fixed 2026-10-09: spent on the first damaging hit of the battle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>258 Adaptation</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Read only among statuses by Unit.resistance. Fixed 2026-10-09.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(sim): the reference party carries its grand sealbook
the reference party carries its grand sealbook (party enchantment and
summon); story bosses checked against the guide

- sheet GrandSealbooks (GameFAQs Grand Sealbooks: Bigfoot, Ghast, Eros
from 36); the summon scales from raw stats, cannot be targeted
(0x43e6d0), so its unknown HP (summon_hp) does not matter - sheet
GuideDifficulty: what the GameFAQs walkthrough says of each story boss
(paraphrased) and a floor of wins per class; tools/guide_curve.py,
docs/generated/GUIDE_CURVE.md: 38 of 40 within, 2 read (C29 heal wall
without ailments, C38 near the floor) - anchors 6/6: the full Queen at
55 (N06) is now met
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -24,6 +24,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditReadings" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GuideDifficulty" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GrandSealbooks" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3486,7 +3488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3758,6 +3760,1257 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>Read only among statuses by Unit.resistance. Fixed 2026-10-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>curve C29</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Calliope heals about 1000 with Splash and 200 a turn with her Carol, as the JP guide says (atwiki dt2-2 page 227): a heal wall. That guide answers it with silence, slow and paralysis; the reference party casts no ailment (its roles have no rule for them) and its physical hits do 100 - 200. 15% at 44, 90% at 54. Theme T07 (ailments).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>curve C38</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>near the floor</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Samael wins 60% at 62 (floor of an easy boss 80%), 100% at 65. The JP guide warns of Chaos Eye (petrification, cured by items in the model) and its resistances (80 to physical) slow a mostly physical party. C38 is a level jump of +7 (CHECKPOINT_LEVELS): a player usually arrives above 62.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Checkpoint</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>What the guide says (paraphrased)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Wanton Witch</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>a total pushover that dies fast to skills</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Ruined Shrine Cave</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mad Catter (miniboss)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ultra weak, dies in one or two turns</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mt. Kongol Fortress</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bigfoot</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nothing special, though a strong physical attacker for a party that rushed</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mt. Kongol Fortress</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mad Catter x3 (miniboss)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>still weak; not too hard once one falls</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mt. Kongol Fortress</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mad Catter</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pretty strong but not deadly; keep the front member healed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mt. Kongol Fortress</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ghast</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>nothing special: heal as needed and use skills</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Tower of Wind</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sorrowful Songstress</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>nothing too dangerous with the wind aura disabled at the shrine; a wipe otherwise</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Tower of Wind</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Doll (miniboss)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>a pushover</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Vrachia Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cupid</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>low damage, not too dangerous</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Vrachia Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Countess of Vrachia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>not too dangerous unless she keeps her dolls up</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Vrachia Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Heqet</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>no trouble with a healing Bard</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dragon Palace</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Boozehound Samurai</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>buffs herself: remove the buffs</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dragon Palace</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Eros</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>two easy companions to rush first</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dragon Palace</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Oh-So-Hime</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>her water line attack can be deadly</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dragon Palace</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Warden of the Wall</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>a bit easier than the previous boss</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Rousset Royal Villa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Molle</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>double physical damage square: squishy members can be one-shot</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Rousset Royal Villa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Agent M</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>take the companions down first</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Rousset Royal Villa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>True Queen Eltricia</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>a very strong boss with two actions a turn; can overwhelm a healing Bard below about level 27</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Rousset Royal Villa</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Siesta</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>sleep plus instant death on sleepers: luck plays a part</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Khorramshahr Outskirts + Altar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Big Bad Beard (miniboss)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>a pushover</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Khorramshahr Outskirts + Altar</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Trafficker Twinny</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>the boss itself poses little danger</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Khorramshahr Outskirts + Altar</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Therian wave, Maerchen Little</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>the wave is weak; the boss is resistant to earth</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Khorramshahr Outskirts + Altar</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Afanc</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>a very easy boss</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Temple of Wrappl</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Martial Artist</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nothing special, should pose no challenge</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Temple of Wrappl</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>C26</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Michelle, Beatrice</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>each a tier behind what the party has faced</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Temple of Wrappl</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>C27</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Forest Guardian x2 (miniboss)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>strong for their low HP but no big problem</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Prizren Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>C28</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Spirit of Mag Mell</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>a big rise in HP; remove her buff at half HP</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Prizren Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>C29</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Calliope</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>somewhat easier than the previous boss</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Prizren Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>C29a</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Dragon Papi</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>one of the toughest fights so far: no magic zone, heal with items</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Prizren Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>C30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Heartless Avenger x2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>two fights in a row; the second is faster and stronger</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Prizren Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>C31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Tres Durian, Mangos Queen</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>weak alone, the difficulty is the two together</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Prizren Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>C32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Moby Dick</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>a pushover overall</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Actim Castle</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>C33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Death Cataphract</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>sturdy against physical but not dangerous</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Actim Castle</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>C34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Queen of Darkness (weakened)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>a relative pushover with the energy feeds destroyed</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Actim Castle</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>C35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Scanner</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>a caster in a magic enhancement zone: massive damage</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dreamscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>C36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Demon God Fried</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>nothing too special</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dreamscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>C37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Iron Maiden</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>kills a member easily but rarely matters if the party keeps reviving</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mage city Gruneworth</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>C38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Samael</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>not too hard of a boss</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), First Sealbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>C39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Melek Taus</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>nothing too dangerous once the zone aura is removed</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), First Sealbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>C40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Demiurge, Atialuco</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>the first melts; the second is more dangerous but most of its damage is not big</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), First Sealbook</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>From checkpoint</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Sealbook</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>833</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bigfoot</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Grand Sealbooks: the first grand sealbook, won from Bigfoot (C03); its summon fights beside the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>913</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Ghast</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Grand Sealbooks: Ghast, the best book up to level 36 at least (damage +10% at full HP, a strong attacker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>760</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Eros</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Grand Sealbooks: Eros, the best summon from level 36 for the rest of the game (turn skips, ailments); C25 is the first checkpoint at 36</t>
         </is>
       </c>
     </row>
@@ -4899,7 +6152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5387,6 +6640,86 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>choice</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>guide_easy_min_won</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>a boss the guide calls easy: the reference party at the reference level wins at least this share (tools/guide_curve.py)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09: the user asked to use the difficulty the guide gives each boss as a point of comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>guide_normal_min_won</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>a boss the guide calls normal</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09: the user asked to use the difficulty the guide gives each boss as a point of comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>guide_hard_min_won</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>a boss the guide calls hard</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09: the user asked to use the difficulty the guide gives each boss as a point of comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>summon_hp</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>9999</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>HP of a summon: not read (docs/FORMULAS.md 11, open); it does not matter in battle because no action can pick a summon (Battle.targetable, 0x43e6d0)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sim): doll actions aimed at the party
doll actions aimed at the party, random results that strike the party,
fixed heal; audit of every active skill

- Catalina healed and Perdurabo cured the doll itself: now the member
lowest in HP and two ailing members (GameFAQs Spieler page, atwiki dt2-2
page 146; setting doll_cure_targets) - hits and ailments of an action
aimed at its own side or at everyone now land there (Magic Box punch and
instant death on the user, Showtime stun, sleep and half HP on the
party; atwiki dt2-2 pages 132, 148); an ailment counts whatever the kind
of its slot; effect 9 alone is a fixed heal - sim_audit actives [k/n]:
235 active skills performed into a prepared battle, effects checked; 23
of 23 flagged rows read; anchors 6/6, guide curve 38/40 with 2 read
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -3488,7 +3488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3794,6 +3794,227 @@
       <c r="C18" t="inlineStr">
         <is>
           <t>Samael wins 60% at 62 (floor of an easy boss 80%), 100% at 65. The JP guide warns of Chaos Eye (petrification, cured by items in the model) and its resistances (80 to physical) slow a mostly physical party. C38 is a level jump of +7 (CHECKPOINT_LEVELS): a player usually arrives above 62.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>125 Magic Box Effect</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The empty result of Magic Box: nothing happens (atwiki dt2-2 page 132).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>140 Showtime Effect</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>The empty result of Showtime: nothing happens (atwiki dt2-2 page 148).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>137 Showtime Effect</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Enemies flee (432) only where running away is allowed: random battles (FORMULAS 12.10); the audit battle is not one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>217 Shadow Sew</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>It lands only on a target of lower level than the user (Battle.after_hit, Shadow Sew compares levels); the audit dummy is level 90 like the user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>233 Soul Eater</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Chance: the spell hits about one time in three against the level 90 dummy and kills 12% of those; a probe of 40 casts saw 2 deaths in 15 hits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>240 Arcane Shield</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>The counter of the Arcane Shield passive: its damage is a share of the damage the bearer took (FORMULAS 12.13); performed alone it has nothing to send back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fixed 2026-10-09 doll targets</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Catalina healed and Perdurabo cured the doll itself (an ally pick with no target): now the member lowest in HP and two ailing members (GameFAQs Spieler page; atwiki dt2-2 page 146).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>fixed 2026-10-09 own-side results</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Hits and ailments landed only on opponents: the random results aimed at the party (Magic Box punch and instant death on the user, Showtime stun, sleep and half HP on every ally) did nothing; Magic Box HP 200 to the party (effect 9 alone) healed nothing (atwiki dt2-2 pages 132, 148).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>86 Materialize</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Effect 84 acts only on an enemy that can be materialized and is below half HP (Battle.after_hit); the dummy is neither.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>105 Perdurabo's Action</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Performed by a member it cures the member, who carries no ailment; as the action of the doll it cures two ailing members (fixed 2026-10-09 doll targets).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>114 Roulette Circus Effect</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>A Roulette result that heals the enemies (effect 128 on random enemies); the dummies are at full HP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>116 Roulette Circus Effect</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>The empty result of Roulette Circus: nothing happens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>119 Magic Box Effect</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Effect 425 ends the chants, songs, dances and dolls of everyone (atwiki dt2-2 page 132); nobody performs one in the audit battle.</t>
         </is>
       </c>
     </row>
@@ -6152,7 +6373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6720,6 +6941,26 @@
       <c r="D28" t="inlineStr">
         <is>
           <t>model choice 2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>doll_cure_targets</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>members whose ailments the doll Perdurabo cures on each of its turns</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Class Skill info - Spieler: two allies per doll turn); atwiki dt2-2 page 146 (味方二人の状態異常を回復)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sim): the Samurai wields a katana
the Samurai wields a katana; Berserk, High Risk High Return, Parry and
Cover rules; every unused skill classified and read

- attacker role: Tachi|Claymore (atwiki dt2-2 page 134: the katana
class; her own skills need one); Geo Break and Sharp Stab out of plans
whose weapon cannot use them - rules: attacker Berserk; joker High Risk
High Return before Trump Card (page 148: Trump Card lasts to the next
turn); valkyrie Parry and Cover on bosses (GameFAQs Recommended Party) -
sim_audit usage [k/n]: each unused skill with its reason (dominated with
the figure, no rule, weapon, situational); 117 of 117 flagged rows read.
Open: no role casts ailments on enemies (theme T07)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -3488,7 +3488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4015,6 +4015,669 @@
       <c r="C31" t="inlineStr">
         <is>
           <t>Effect 425 ends the chants, songs, dances and dolls of everyone (atwiki dt2-2 page 132); nobody performs one in the audit battle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>usage attacker | War Cry</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>redundant</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>The party ATK buff is kept by the Valkyrie (rule status:161); a second giver adds nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>usage dark lord | War Cry</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>redundant</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>The party ATK buff is kept by the Valkyrie (rule status:161); a second giver adds nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>usage tank | War Cry</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>redundant</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>The party ATK buff is kept by the Valkyrie (rule status:161); a second giver adds nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>usage tank | Cover</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>The tank draws attacks with Provoke (rule status:170); Cover is the Valkyrie's prebuff (rule boss status:171).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>usage diva | Blissful Chorale</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Her song slots hold the heal song and the speed song (rules status:215, 217, GameFAQs faqs/80834 Recommended Party).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>usage maid | Blissful Chorale</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Her song slot holds Replenishing Carol (rule status:215).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>usage maid | Concentration Prelude</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Her song slot holds Replenishing Carol (rule status:215).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>usage maid | Lightning March</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Her song slot holds Replenishing Carol; the speed song is the Diva's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>usage dolls | Catalina</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>doll order</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>The doll rule fills the slots in its order (Spartan, Catalina, Oracles); the first ones fill them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>usage dolls | Oracles</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>doll order</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>The doll rule fills the slots in its order; GameFAQs faqs/80834 Spieler page: "don't bother" with Oracles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>usage soul summoner | Catalina</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>doll order</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>The doll rule fills both slots with Mercidarian and Spartan first (GameFAQs faqs/80834: Mercidarian by far the best doll).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>usage soul summoner | Oracles</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>doll order</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>The doll rule fills both slots with Mercidarian and Spartan first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>usage soul summoner | Musiy</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>doll order</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>The doll rule fills both slots with Mercidarian and Spartan first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>usage soul summoner | Perdurabo</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>doll order</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>The doll rule fills both slots first; the cure doll is not in its order (the party cures with items).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>usage etoile | Alluring Samba</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka (rules status:195, 201).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>usage etoile | Debilitating Salsa</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>usage etoile | Emaciating Hopak</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>usage etoile | Gloomy Tango</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>usage etoile | Gravitating Polka</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>slots</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Her two dance slots hold Fascinating Waltz and Dumbing Mazurka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>usage etoile | Clean</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>No rule; a minor buff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>usage healer | Insurance</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>No rule for protective prebuffs; the healer heals, cures and dispels first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>usage healer | Moon Curtain</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>No rule for protective prebuffs; the healer heals, cures and dispels first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>usage valkyrie | Material Guard</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>A late prebuff of her plan; no rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>usage valkyrie | Moon Curtain</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>A late prebuff of her plan (learned near 90); no rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>usage valkyrie | Protect</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>A late prebuff of her plan (learned near 90); no rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>usage magical princess | Accelerator</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>A rule for it made her spend every turn on single-target buffs (2026-10-09); left out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>usage magical princess | Cover</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Cover is the Valkyrie's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>usage magical princess | Magic Barrier</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>No rule; a minor buff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>usage papillon | High Risk, High Return</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 Recommended Party uses it only to act at once against familiars; her damage is Rose Queen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>usage shooter | Aim</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>No rule; an accuracy buff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>usage sage | Bash Guard</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>A guard against one kind of blow: no rule picks it by the enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>usage sage | Slash Guard</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>A guard against one kind of blow: no rule picks it by the enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>usage sage | Stab Guard</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>A guard against one kind of blow: no rule picks it by the enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>usage sage | Sleep</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ailments</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>No role casts ailments on enemies: open point of theme T07.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>usage sage | Silence</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>ailments</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>No role casts ailments on enemies: open point of theme T07 (the JP guide names silence against Calliope, C29).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>usage kunoichi | Shadow Sew</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ailments</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>No role casts ailments on enemies: open point of theme T07.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>usage kunoichi | Light Scroll</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ailments</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>An accuracy debuff on enemies: no rule (theme T07).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>usage kunoichi | Evade</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>policy gap</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>No rule; an evasion buff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>usage treasure hunter | Chain Spike</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>role choice</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>It needs a bow or a gun; the role fights with a dagger (GameFAQs faqs/80834: she moves to a gun late).</t>
         </is>
       </c>
     </row>
@@ -6975,7 +7638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7078,37 +7741,37 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:26</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 123: Berserk is the core of the Berserker line, kept up by the Samurai who comes from it</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dark lord</t>
+          <t>attacker</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -7119,21 +7782,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -7144,21 +7807,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the dispel on Berserker, for boss buffs</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
@@ -7169,21 +7832,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>status:191</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the dispel on Berserker, for boss buffs</t>
         </is>
       </c>
     </row>
@@ -7194,7 +7857,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -7203,12 +7866,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>status:26</t>
+          <t>status:191</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "once you get berserk you should also upkeep berserk"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "the rotation is Power Charge &gt; Nuke"</t>
         </is>
       </c>
     </row>
@@ -7219,7 +7882,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -7228,37 +7891,37 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:26</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "once you get berserk you should also upkeep berserk"</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>diva</t>
+          <t>dark lord</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -7269,21 +7932,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: First Aid or an item in an emergency</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items when a member falls</t>
         </is>
       </c>
     </row>
@@ -7294,21 +7957,21 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "upkeeps Heal/Speed song in boss battles"; the heal song first</t>
+          <t>GameFAQs faqs/80834, Recommended Party: First Aid or an item in an emergency</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7982,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -7328,12 +7991,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>status:217</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the speed song</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "upkeeps Heal/Speed song in boss battles"; the heal song first</t>
         </is>
       </c>
     </row>
@@ -7344,21 +8007,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.35</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>tp:0.35</t>
+          <t>status:217</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "helps manage the party TP with cook and self sacrifice"</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the speed song</t>
         </is>
       </c>
     </row>
@@ -7369,46 +8032,46 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.35</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.35</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "helps manage the party TP with cook and self sacrifice"</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dolls</t>
+          <t>diva</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>doll_slot_free</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>doll:Spartan|Catalina|Oracles</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 131; a free doll slot is filled (two with Double Puppet, page 146); GameFAQs Class Skill info - Spieler: Spartan first, Oracles "don't bother"</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -7419,46 +8082,46 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>doll:Spartan|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 131; a free doll slot is filled (two with Double Puppet, page 146); GameFAQs Class Skill info - Spieler: Spartan first, Oracles "don't bother"</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>etoile</t>
+          <t>dolls</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -7469,21 +8132,21 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>status:195</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fascinating Waltz on the enemies</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -7494,7 +8157,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -7503,12 +8166,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>status:201</t>
+          <t>status:195</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Dumbing Mazurka on the enemies</t>
+          <t>Fascinating Waltz on the enemies</t>
         </is>
       </c>
     </row>
@@ -7519,21 +8182,21 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.35</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>tp:0.35</t>
+          <t>status:201</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Cook</t>
+          <t>Dumbing Mazurka on the enemies</t>
         </is>
       </c>
     </row>
@@ -7544,46 +8207,46 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.35</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.35</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Cook</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>healer</t>
+          <t>etoile</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -7594,16 +8257,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.6</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>heal:0.6</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7619,16 +8282,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ally_ailing</t>
+          <t>ally_hp_below:0.6</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>cure</t>
+          <t>heal:0.6</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7644,16 +8307,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>ally_ailing</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>cure</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7669,46 +8332,46 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>joker</t>
+          <t>healer</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -7719,21 +8382,21 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>status:48</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Trump Card on bosses (page 148)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -7748,53 +8411,53 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:48</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Trump Card on bosses (page 148)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>kunoichi</t>
+          <t>joker</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>status:101</t>
+          <t>status:26</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Shadow Clone kept up (page 142)</t>
+          <t>atwiki dt2-2 page 132: High Risk, High Return is the main skill of the Trickster line, beside Trump Card; cast before Trump Card, whose effect lasts only to the next turn (atwiki dt2-2 page 148)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>kunoichi</t>
+          <t>joker</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -7815,7 +8478,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>kunoichi</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -7823,24 +8486,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>status:101</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>Shadow Clone kept up (page 142)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>kunoichi</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -7865,7 +8528,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -7873,24 +8536,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>status:189</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Magical Change kept up (page 137)</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -7915,7 +8578,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -7923,24 +8586,24 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:189</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>Magical Change kept up (page 137)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -7948,17 +8611,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.5</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -7969,21 +8632,21 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.4</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>tp:0.4</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
@@ -7994,21 +8657,21 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_hp_below:0.5</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 129: Replenishing Carol</t>
+          <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
         </is>
       </c>
     </row>
@@ -8019,57 +8682,57 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.4</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.4</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 120</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Resurrect or items</t>
+          <t>atwiki dt2-2 page 129: Replenishing Carol</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -8078,12 +8741,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>the heal song kept up</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8094,21 +8757,21 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>War Cry kept up</t>
+          <t>Resurrect or items</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8782,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -8128,62 +8791,62 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>the heal song kept up</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>War Cry kept up</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8194,71 +8857,71 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>heals when the party is low</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
         </is>
       </c>
     </row>
@@ -8269,21 +8932,21 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Dispel against boss buffs</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -8294,21 +8957,21 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up)</t>
+          <t>heals when the party is low</t>
         </is>
       </c>
     </row>
@@ -8319,21 +8982,21 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>status:162</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138 (Circle Protect kept up)</t>
+          <t>Dispel against boss buffs</t>
         </is>
       </c>
     </row>
@@ -8344,7 +9007,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -8353,12 +9016,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>status:163</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Sun Veil kept up</t>
+          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up)</t>
         </is>
       </c>
     </row>
@@ -8369,7 +9032,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -8378,12 +9041,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>status:172</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Amplify kept up</t>
+          <t>atwiki dt2-2 page 138 (Circle Protect kept up)</t>
         </is>
       </c>
     </row>
@@ -8394,7 +9057,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -8403,12 +9066,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>status:168</t>
+          <t>status:163</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Accelerator (one ally, 3 turns) after the party-wide buffs</t>
+          <t>Sun Veil kept up</t>
         </is>
       </c>
     </row>
@@ -8419,7 +9082,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -8428,23 +9091,23 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:172</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Amplify kept up</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>shooter</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -8453,48 +9116,48 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:168</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Accelerator (one ally, 3 turns) after the party-wide buffs</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>doll_slot_free</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>shooter</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -8515,7 +9178,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -8523,24 +9186,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -8553,12 +9216,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>status:170</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8569,21 +9232,21 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
@@ -8594,7 +9257,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -8603,12 +9266,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>status:162</t>
+          <t>status:170</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
+          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
         </is>
       </c>
     </row>
@@ -8619,71 +9282,71 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 133</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8694,21 +9357,21 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
         </is>
       </c>
     </row>
@@ -8719,71 +9382,71 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
         </is>
       </c>
     </row>
@@ -8794,21 +9457,21 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -8819,21 +9482,21 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>status:183</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
@@ -8844,21 +9507,21 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
         </is>
       </c>
     </row>
@@ -8869,19 +9532,119 @@
         </is>
       </c>
       <c r="B76" t="n">
+        <v>4</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>status:183</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>5</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>status:161</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
         <v>6</v>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>status:180</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>7</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>status:171</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>8</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
         </is>
@@ -9078,7 +9841,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Claymore|Tachi</t>
+          <t>Tachi|Claymore</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -9104,7 +9867,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>War Cry; Raging Smash; Sword Mastery; Double Attack; Aura Eliminate; Berserk; Frost Slash; Geo Break; Katana Mastery; Moonlight Purgatory; Onikagura; Triple Attack; Armor Penetration; Mind's Eye</t>
+          <t>War Cry; Raging Smash; Sword Mastery; Double Attack; Aura Eliminate; Berserk; Frost Slash; Katana Mastery; Moonlight Purgatory; Onikagura; Triple Attack; Armor Penetration; Mind's Eye</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -9114,7 +9877,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 123, 134</t>
+          <t>atwiki dt2-2 pages 123, 134; page 134: the Samurai is the katana class (her own skills need one); the first piece of the list her class can wear is taken</t>
         </is>
       </c>
     </row>
@@ -9356,7 +10119,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Sharp Stab; Poison Shot; Bow Mastery; Freeze Shot; Arrow Rain; Aim; Chain Spike; Spiral Arrow; Divine Cannon; Warning Shot; Support Shot</t>
+          <t>Poison Shot; Bow Mastery; Freeze Shot; Arrow Rain; Aim; Chain Spike; Spiral Arrow; Divine Cannon; Warning Shot; Support Shot</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(sim): an ailment rule (act_ailment)
an ailment rule (act_ailment): the Sage casts slow, silence or sleep and
the Kunoichi Shadow Sew on bosses when the roll reaches
ailment_min_chance
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -7036,7 +7036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7624,6 +7624,26 @@
       <c r="D29" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (Class Skill info - Spieler: two allies per doll turn); atwiki dt2-2 page 146 (味方二人の状態異常を回復)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ailment_min_chance</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>a role casts an ailment on an enemy only when its roll has at least this chance against the enemy's resistance (sim/policy.py act_ailment)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09: a player does not spend a turn on a roll that likely fails</t>
         </is>
       </c>
     </row>
@@ -7638,7 +7658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8407,7 +8427,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -8416,12 +8436,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>status:48</t>
+          <t>status:26</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Trump Card on bosses (page 148)</t>
+          <t>atwiki dt2-2 page 132: High Risk, High Return is the main skill of the Trickster line, beside Trump Card; cast before Trump Card, whose effect lasts only to the next turn (atwiki dt2-2 page 148)</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8452,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -8441,12 +8461,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>status:26</t>
+          <t>status:48</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 132: High Risk, High Return is the main skill of the Trickster line, beside Trump Card; cast before Trump Card, whose effect lasts only to the next turn (atwiki dt2-2 page 148)</t>
+          <t>Trump Card on bosses (page 148)</t>
         </is>
       </c>
     </row>
@@ -8511,42 +8531,42 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>ailment:123</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 142: Shadow Sew, the ailment of the Kunoichi; it lands only on a lower level target</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>mage</t>
+          <t>kunoichi</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8557,32 +8577,32 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>magical princess</t>
+          <t>mage</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -8591,12 +8611,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>status:189</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Magical Change kept up (page 137)</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8607,7 +8627,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -8616,37 +8636,37 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:189</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Magical Change kept up (page 137)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>maid</t>
+          <t>magical princess</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8657,21 +8677,21 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
@@ -8682,21 +8702,21 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.4</t>
+          <t>ally_hp_below:0.5</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>tp:0.4</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 120</t>
+          <t>atwiki dt2-2 page 120: the Maid restores HP and TP at no cost</t>
         </is>
       </c>
     </row>
@@ -8707,21 +8727,21 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.4</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>tp:0.4</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 129: Replenishing Carol</t>
+          <t>atwiki dt2-2 page 120</t>
         </is>
       </c>
     </row>
@@ -8732,7 +8752,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -8741,37 +8761,37 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 129: Replenishing Carol</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>mistress</t>
+          <t>maid</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Resurrect or items</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8782,21 +8802,21 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>status:215</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>the heal song kept up</t>
+          <t>Resurrect or items</t>
         </is>
       </c>
     </row>
@@ -8807,7 +8827,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -8816,12 +8836,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>status:215</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>War Cry kept up</t>
+          <t>the heal song kept up</t>
         </is>
       </c>
     </row>
@@ -8832,7 +8852,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -8841,37 +8861,37 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>War Cry kept up</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>papillon</t>
+          <t>mistress</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -8882,21 +8902,21 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -8907,46 +8927,46 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>sage</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the best area attack and the damage of the party</t>
         </is>
       </c>
     </row>
@@ -8957,21 +8977,21 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>heals when the party is low</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -8982,21 +9002,21 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>enemy_buffed</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>dispel</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Dispel against boss buffs</t>
+          <t>heals when the party is low</t>
         </is>
       </c>
     </row>
@@ -9007,21 +9027,21 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>enemy_buffed</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>dispel</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up)</t>
+          <t>Dispel against boss buffs</t>
         </is>
       </c>
     </row>
@@ -9032,21 +9052,21 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>boss</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>status:162</t>
+          <t>ailment:122;117;116</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138 (Circle Protect kept up)</t>
+          <t>atwiki dt2-2 page 138: the Sage supports with ailment spells; slow, silence and sleep in that order (page 227 names slow and silence against the heal wall of Calliope)</t>
         </is>
       </c>
     </row>
@@ -9057,7 +9077,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -9066,12 +9086,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>status:163</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Sun Veil kept up</t>
+          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up)</t>
         </is>
       </c>
     </row>
@@ -9082,7 +9102,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -9091,12 +9111,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>status:172</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Amplify kept up</t>
+          <t>atwiki dt2-2 page 138 (Circle Protect kept up)</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9127,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -9116,12 +9136,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>status:168</t>
+          <t>status:163</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Accelerator (one ally, 3 turns) after the party-wide buffs</t>
+          <t>Sun Veil kept up</t>
         </is>
       </c>
     </row>
@@ -9132,7 +9152,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -9141,23 +9161,23 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:172</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Amplify kept up</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>shooter</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -9166,48 +9186,48 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>status:168</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>Accelerator (one ally, 3 turns) after the party-wide buffs</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>sage</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>doll_slot_free</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>soul summoner</t>
+          <t>shooter</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -9228,7 +9248,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -9236,24 +9256,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>doll_slot_free</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>doll:Mercidarian|Spartan|Musiy|Catalina|Oracles</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
+          <t>atwiki dt2-2 pages 131, 146: both doll slots kept filled; GameFAQs Class Skill info - Spieler: Mercidarian by far the best doll</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>soul summoner</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -9266,12 +9286,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>status:170</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -9282,21 +9302,21 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 133</t>
+          <t>GameFAQs faqs/80834 (balance_criteria F01): a party holds a Maid, a dispeller and a healer</t>
         </is>
       </c>
     </row>
@@ -9307,7 +9327,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -9316,12 +9336,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>status:162</t>
+          <t>status:170</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
+          <t>atwiki dt2-2 page 133: the Valkyrie draws attacks as the wall of the party</t>
         </is>
       </c>
     </row>
@@ -9332,71 +9352,71 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>the mean damage per time of every skill</t>
+          <t>atwiki dt2-2 page 133</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>status:162</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
+          <t>atwiki dt2-2 page 122: the Paladin uses herself as the shield of the party (Protect kept up on the weakest member)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>treasure hunter</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>the mean damage per time of every skill</t>
         </is>
       </c>
     </row>
@@ -9407,21 +9427,21 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ally_hp_below:0.35</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>heal:0.35</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "can help with items in emergency situations"</t>
         </is>
       </c>
     </row>
@@ -9432,71 +9452,71 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>damage</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ally_down</t>
+          <t>ally_hp_below:0.35</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>revive</t>
+          <t>heal:0.35</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>items when a member falls</t>
+          <t>GameFAQs faqs/80834, Recommended Party: items in an emergency</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>valkyrie</t>
+          <t>treasure hunter</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ally_tp_below:0.15</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>tp:0.15</t>
+          <t>damage</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
+          <t>GameFAQs faqs/80834, Recommended Party: Pursuit Stab as the core</t>
         </is>
       </c>
     </row>
@@ -9507,21 +9527,21 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>party_hp_below:0.5</t>
+          <t>ally_down</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>heal:0.5</t>
+          <t>revive</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
+          <t>items when a member falls</t>
         </is>
       </c>
     </row>
@@ -9532,21 +9552,21 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>ally_tp_below:0.15</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>status:183</t>
+          <t>tp:0.15</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
+          <t>a fruit when a member runs dry (the items of the sheet Kit)</t>
         </is>
       </c>
     </row>
@@ -9557,21 +9577,21 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>party_hp_below:0.5</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>status:161</t>
+          <t>heal:0.5</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
+          <t>GameFAQs faqs/80834, Recommended Party: "in serious bosses she should usually be supporting"</t>
         </is>
       </c>
     </row>
@@ -9582,21 +9602,21 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>status:180</t>
+          <t>status:183</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+          <t>GameFAQs faqs/80834, Recommended Party: the guard buffs of the party</t>
         </is>
       </c>
     </row>
@@ -9607,21 +9627,21 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>status:171</t>
+          <t>status:161</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+          <t>GameFAQs faqs/80834, Recommended Party: War Cry maxed early</t>
         </is>
       </c>
     </row>
@@ -9632,19 +9652,69 @@
         </is>
       </c>
       <c r="B80" t="n">
+        <v>6</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>status:180</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>7</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>status:171</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834, Recommended Party: the Valkyrie prebuffs Parry and Cover in hard fights</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
         <v>8</v>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
         </is>

</xml_diff>

<commit_message>
feat: every class measured at its stage
every class measured at its stage (tools/class_stages.py, sheets
ClassStages, ClassKinds); Action effects cached (2x faster); parallel
runs

- base C03-C06, intermediate C10-C18, advanced C22-C40, late P08-P24;
each of 19 roles in the last place of the reference party, 15 fights;
attackers judged by the length of won fights, supports and tanks by wins
in the contested fights; 65 of 76 rows within, 11 slow or weak; P17 lost
by every class (to read) - Action.effects worked out once per action: a
stage run from over 20 minutes to under 7 with 6 processes
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -26,6 +26,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditReadings" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GuideDifficulty" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GrandSealbooks" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClassStages" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClassKinds" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7030,13 +7032,712 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Checkpoints</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Levels</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C03; C05; C06</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5 - 9</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-09: each class measured at the stage where it is played, against several bosses of it; the class path changes at 15 and 30 (scenario.class_path)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C10; C13; C18</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>15 - 27</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-09: each class measured at the stage where it is played, against several bosses of it; the class path changes at 15 and 30 (scenario.class_path)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C22; C29; C34; C40</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>33 - 64</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-09: each class measured at the stage where it is played, against several bosses of it; the class path changes at 15 and 30 (scenario.class_path)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>late</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>P08; P17; P24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>72 - 90</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>the user, 2026-10-09: each class measured at the stage where it is played, against several bosses of it; the class path changes at 15 and 30 (scenario.class_path)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Maid</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p120: the unsung pillar, effects without TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bard</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p129: her songs strengthen and heal the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dancer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p130: debuffer through dances</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Priestess</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p126: rear support excelling at healing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Enchantress</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p125: support through elements, ailments and buffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Diva</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p128</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Etoile</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p147</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Bishop</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p139: the healing specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sage</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p138: support that raises allies</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Paladin</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p122: uses herself as the shield of the party</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Valkyrie</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md; atwiki dt2-2 p133: protects her allies (guard skills, Cover, Parry)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Fighter</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Berserker</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Samurai</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Dark Lord</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Magic User</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sorceress</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Witch</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Magical Princess</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Scout</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Archer</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Treasure Hunter</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Kunoichi</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mistress</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Spieler</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Doll Master</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Trickster</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Soul Summoner</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Papillon</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Joker</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>docs/CLASS_IDENTITY.md (role: damage)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7644,6 +8345,86 @@
       <c r="D30" t="inlineStr">
         <is>
           <t>model choice 2026-10-09: a player does not spend a turn on a roll that likely fails</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>class_slow_ratio</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>a role whose fights last more than this times the median of the roles at its stage is slow (tools/class_stages.py)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09: the measure has about 5% of noise at 15 battles; 15% is a gap the player feels</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>parallel_workers</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>processes a tool may run at once (tools/class_stages.py all): each takes about 80 MB; 12 cores, about 6 GB free</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09: the user asked for faster runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>parallel_slices</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>slices of the roles of one checkpoint, so that a long checkpoint is spread over several processes</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09: the user asked for faster runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>class_weak_wins</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>a role whose share of wins in the contested fights of its stage is this much below the median is weak (tools/class_stages.py)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sim): the altars and shrines a player uses before a boss
the altars and shrines a player uses before a boss (sheet ZoneChanges):
C07 wind shrine, C39 wind and earth altar, P17 magic boost turned to
water (GameFAQs walkthrough; atwiki dt2-2 page 326)

C07 85 -> 100%, C39 75 -> 90%; P17 still lost: Last Judgment's damage
checked against the code (enemy attack power, 0x44b47a - 0x44b4a1), its
AI script and its speed
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -28,6 +28,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GrandSealbooks" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClassStages" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClassKinds" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ZoneChanges" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7731,6 +7732,170 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>New slot</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>St02_0070</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sorrowful Songstress (C07)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Tower of Wind: with the wind aura disabled at the shrine of map 7 she has nothing too dangerous</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>St02_0070</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>41</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sorrowful Songstress (C07)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Tower of Wind (the cell carries the wind slot twice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>St15_1120</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>41</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Melek Taus (C39)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), First Sealbook: the altar of the west side disables the wind and earth aura, useful against the boss</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>St15_1120</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>41</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Melek Taus (C39)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), First Sealbook (the earth slot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>St23_0060</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>41</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Last Judgment (P17)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Plains of Light part 1: the altar near the entrance changes the magic damage boost into an element; water, the weakest point of the boss, who has no water attack</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
data: the 30 postgame bosses against the GameFAQs walkthrough
the 30 postgame bosses against the GameFAQs walkthrough: 9 within, 21
below (the reference party lacks the unique postgame gear the guide
uses)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -4695,7 +4695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5802,6 +5802,816 @@
       <c r="E41" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834 (Hentaicheg), First Sealbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Aradia (1st fight)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>super easy, there to unlock the postgame</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Iktomi</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>pretty weak aside of a TP drain, very squishy</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Hell's Hole</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Aradia (2nd fight)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>stronger than before, a few strong physical nukes</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Hell's Hole</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sukuna-Hikona</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>very squishy to physical for this point, falls fast</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Hell's Hole</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Euthys</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>strong stats but skills not too dangerous; the party should be ready by now</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Casino Esperanza; GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Overdue</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>at low HP a long chant of 2,000 fixed damage to everyone, very likely a game over</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Prizren Woods</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Royal Villa, three bosses</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>level about 60 and about 10k HP each; burst them in the no magic zone</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Qitian Dasheng</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>a very weak boss in general</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Casino Esperanza</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Azathoth</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>a fast caster with dark aura, two weak companions</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Casino Esperanza</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Kuchinawa</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>stronger than its level but a burst fight the Dark Lord can end at once</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Aradia (3rd fight)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>stronger than her level</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Genbu</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>massive defence and resistances, counters short range: an annoying fight</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Matrix; GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Nuwa</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>an annoying fight</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Murasaki Shikibu</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>level 82, taken once the quest appears</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Aradia (4th fight)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>stronger than her level, in a physical defence zone</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Aradia (5th fight)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>not harder in stats; instant kill chances on her skills</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Last Judgment</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>very weak stats for such a late boss, but a long chant of 2,000 to everyone (atwiki dt2-2 page 326: fairly easy once the altar turns the zone to a useful element)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Plains of Light part 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Aradia (6th fight)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>slightly better stats, dark aura</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Three goddesses</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>pretty tough: the three together are really strong</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Plains of Light part 1; GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Crom Cruach (weakened superboss)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>a weakened superboss</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>P21</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Ria the Farsighted</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>a pushover overall</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dreamscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>P22</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Chika the Impenetrable</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>close to the hardest boss of the game for a physical team without preparation</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dreamscape</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>P23</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Samael (Dreamscape)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>one of the level 85 - 88 bosses of the depth</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>P24</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Aradia (7th fight)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>level 88</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Mil the Overlord</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>a total pushover</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mage city Gruneworth</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Lina the Statuesque</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>a total pushover; only the party profits from the zone</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mage city Gruneworth</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>P27</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Melek Taus (Gruneworth)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>lots of HP in a zone doubling both kinds of damage</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mage city Gruneworth</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>P28</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Hell's Angel</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>level 92 boss</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>P29</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Panagia (weakened)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>very weak for the level, a total joke when reached</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>P30</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Lolo and Tenerezza (weakened superboss)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>a weakened superboss</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Quick Summary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sim): the postgame party wears the unique gear and the personal
the postgame party wears the unique gear and the personal sealbooks of
the guide (sheets UniqueGear, PersonalSealbooks)

Pulse Blaster, Psychogun, Kuchinawa's Cleaver, God Destroyer, Llyr's
Spear, Edge of Tartarus, Phantom Menace, Professor's Flute, Sword-Sage's
Eyepatch; Persephone, Demi Lich, Himiko, each from the checkpoint the
GameFAQs guide gets it. Postgame bosses within the guide's class: 9 ->
13 of 30; story 38 of 40 unchanged; anchors 6/6
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -29,6 +29,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClassStages" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClassKinds" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ZoneChanges" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UniqueGear" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PersonalSealbooks" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8706,6 +8708,833 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Piece</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>From checkpoint</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pulse Blaster</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Casino Esperanza: Euthys (P05) gives a two-handed gun of massive attack, for the Papillon; atwiki dt2-2 page 186 (パルスレーザーガン)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Psychogun</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Matrix map 2 chest (after Genbu, P12): the best one-handed gun, used by the Papillon until a fan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Kuchinawa's Cleaver</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Ruined Shrine Cave: Kuchinawa (P10) drops a pretty good two-handed axe; atwiki dt2-2 page 29 (クチナワの大鉈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>God Destroyer</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>P28</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Mage city Gruneworth: Melek Taus (P27) drops God Destroyer, a one-handed axe</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Llyr's Spear</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>P21</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Hell's Hole: the water spear of the weakened superboss (P20); Gruneworth: recommended against Lina</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Edge of Tartarus</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>P24</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dreamscape: Carmilla (very powerful enemy of the depth, P21 - P23) drops the best dagger, for the Treasure Hunter and the Joker</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>joker</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Edge of Tartarus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>P24</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Dreamscape: Carmilla drops the best dagger, for the Joker</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Phantom Menace</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>P29</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Plains of Light part 2: the best microphone from the Little Mermaid of map 12 on</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Professor's Flute</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot: Gruneworth map 6 chest</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sword-Sage's Eyepatch</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Matrix: a great accessory for physical characters (ATK 30, DEX 20)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Sealbook</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>From checkpoint</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dark lord</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>458</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>papillon</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>458</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>valkyrie</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>458</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>treasure hunter</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>458</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>458</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>joker</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>458</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>458</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>kunoichi</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>458</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mistress</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>458</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>458</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>458</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>458</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Persephone</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Persephone (level 66, sealed in the first postgame dungeon), "can get it early and it is pretty solid forever" for physical roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>diva</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>453</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Demi Lich</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>453</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Demi Lich</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>453</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Demi Lich</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>453</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Demi Lich</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>magical princess</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>453</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Demi Lich</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>maid</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>453</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Demi Lich</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Demi Lich (level 69), "a pretty early sealbook", for the Diva and offensive mages</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>etoile</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>56</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Himiko</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Best in Slot Gear + Sealbooks: Himiko (level 81, a regular monster), top tier for the Etoile</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
data: class stages: the late stage measured on the postgame bosses the
class stages: the late stage measured on the postgame bosses the model
reproduces (P08, P14, P18, P24); the rest of the postgame a known limit
until T08
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -7950,7 +7950,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P08; P17; P24</t>
+          <t>P08; P14; P18; P24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -7960,7 +7960,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>the user, 2026-10-09: each class measured at the stage where it is played, against several bosses of it; the class path changes at 15 and 30 (scenario.class_path)</t>
+          <t>the user, 2026-10-09: only the postgame bosses the model reproduces (within the floor of the GameFAQs class with margin, docs/generated/GUIDE_CURVE.md); the rest of the postgame is a known limit until theme T08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: T07 measure (skill_value.py ailments)
T07 measure (skill_value.py ailments): every hostile skill with and
without, on boss fights and rows of random battles of its stage

Result: the ailments land (Silence 124 of 190 rolls, Slow 237 of 317)
but add nothing: at the reference level the party ends the boss fights
and the rows of random battles with 98 - 99% of its HP, so nothing is
worth disabling. T07 waits for the difficulty (T02, T08)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -9541,7 +9541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10309,6 +10309,26 @@
       <c r="D38" t="inlineStr">
         <is>
           <t>model choice 2026-10-09 for T06</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ailment_chain</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>random battles in a row (HP and TP carried) on which tools/skill_value.py ailments measures each hostile skill</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>model choice 2026-10-09 for T07: a stretch of dungeon between two returns</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the seven parties counted one by one
the seven parties counted one by one, the Plus ones no longer folded
into their archetype
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -9700,7 +9700,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Juggernaut</t>
+          <t>Juggernaut-Plus</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -9754,7 +9754,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Anti-Meta</t>
+          <t>Anti-Meta-Plus</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>

<commit_message>
sim: five parties, the Plus ones in the place of Juggernaut and
five parties, the Plus ones in the place of Juggernaut and Anti-Meta
without a Diva (decided 2026-10-11); boss fit run again
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -9554,7 +9554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9668,108 +9668,54 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Juggernaut</t>
+          <t>Juggernaut-Plus</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Juggernaut</t>
+          <t>Juggernaut-Plus</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>tank; attacker; dark lord; kunoichi; etoile</t>
+          <t>tank; attacker; dark lord; kunoichi; diva</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The five parties of the user (tools/parallel_party_battery.py of commit 864b1e6), by degree of optimisation</t>
+          <t>The same party with a Diva in its last place (commit d25c8ed, 2026-10-11): the archetype with a healer and TP support. It takes the place of the party without a Diva (the user, 2026-10-11): that one ignores the basics, and whoever plays it can swap one member</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Juggernaut-Plus</t>
+          <t>Anti-Meta-Plus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Juggernaut-Plus</t>
+          <t>Anti-Meta-Plus</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>tank; attacker; dark lord; kunoichi; diva</t>
+          <t>magical princess; mistress; soul summoner; dolls; diva</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>The same party with a Diva in its last place (commit d25c8ed, 2026-10-11): the archetype with a healer and TP support</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Anti-Meta</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Anti-Meta</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>magical princess; mistress; soul summoner; joker; dolls</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>The five parties of the user (tools/parallel_party_battery.py of commit 864b1e6), by degree of optimisation</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Anti-Meta-Plus</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Anti-Meta-Plus</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>magical princess; mistress; soul summoner; dolls; diva</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>60%</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>The same party with a Diva in its last place (commit d25c8ed, 2026-10-11): the archetype with a healer and TP support</t>
+          <t>The same party with a Diva in its last place (commit d25c8ed, 2026-10-11): the archetype with a healer and TP support. It takes the place of the party without a Diva (the user, 2026-10-11): that one ignores the basics, and whoever plays it can swap one member</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bosses: C36 classed normal, on what the fight is and what the battery
C36 classed normal, on what the fight is and what the battery wins in
vanilla; reports regenerated
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -5698,12 +5698,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>easy</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>nothing too special</t>
+          <t>nothing too special (said of its mechanics: no trick to learn). Classed normal on 2026-10-11: the fight is 18,000 HP, an action that leaves the whole party at 1 HP about every five units of time (Creation and Destruction, effect 142) and single blows of 600 - 700 (Iron Hammer of Death); in vanilla only one of the five parties of the battery wins 80% of the time</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">

</xml_diff>

<commit_message>
sim: every role eats a TP fruit when a member runs dry
every role eats a TP fruit when a member runs dry, as the roles of the
reference party did; every report replayed

The diagnosis of C32, C36 and C40 showed the parties that failed
fighting on with plain attacks while the eight Fairy Apples of the bag
stayed unused: twelve roles had no such rule. Anchors 6 of 6, curve 37
of 44 within and 0 harder, battery 65 of 85 in vanilla and 76 of 85 on
the variant; Mage-Heavy is above its floor at every boss.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -10682,7 +10682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12766,6 +12766,306 @@
       <c r="E83" t="inlineStr">
         <is>
           <t>GameFAQs faqs/80834, Recommended Party: Daedalus, "one of the best fire and forget nukes"</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>magical princess</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>mistress</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>soul summoner</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>dolls</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>attacker</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>kunoichi</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>shooter</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>joker</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ally_tp_below:0.15</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>tp:0.15</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>a fruit when a member runs dry (the items of the sheet Kit), as the roles of the reference party do: without it these roles left the eight Fairy Apples of the bag unused and fought on with plain attacks (diagnosis of C32, C36 and C40, 2026-10-11)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the mage raises her passives before a second element
the mage raises her passives before a second element, the Sage keeps the
attack buff last; every report replayed

Anchors 6 of 6, curve 37 of 44 within and 0 harder, battery 66 of 85 in
vanilla and 76 of 85 on the variant, no boss admits more. The plan
records what the project saw in the game on 2026-10-11: the patched
program starts, and the three mechanisms nobody had seen on screen work.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -12126,7 +12126,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -12140,7 +12140,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up)</t>
+          <t>atwiki dt2-2 page 138: the Sage raises the abilities of the party (Circle Brave kept up) | last since 2026-10-11: the attack buff serves the fewest members of the parties a Sage is in</t>
         </is>
       </c>
     </row>
@@ -12151,7 +12151,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -12176,7 +12176,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -12201,7 +12201,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -12226,7 +12226,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -13475,7 +13475,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Fireball; Ice Edge; Thunderbolt; Fire Blast; Ice Storm; Magic Mastery; Critical Magic; Concentrate; Crimson Flare; Cocytus; Muon Plasma; Tempest; Gaia Crush; Inferno; Diamond Dust; Meteor; Fast Cast; Economy; Nirvana</t>
+          <t>Fireball; Magic Mastery; Concentrate; Economy; Critical Magic; Thunderbolt; Fast Cast; Ice Edge; Crimson Flare; Muon Plasma; Cocytus; Tempest; Gaia Crush; Fire Blast; Ice Storm; Inferno; Diamond Dust; Meteor; Nirvana</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -13485,7 +13485,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 pages 124, 136; the strongest single spell of each element before the area ones (page 136: the Witch gathers the great single and all-target spells of every element)</t>
+          <t>atwiki dt2-2 pages 124, 136; the strongest single spell of each element before the area ones (page 136: the Witch gathers the great single and all-target spells of every element). Order of 2026-10-11 (choice): the passives of the caster (damage, concentration, TP cost) before a second and a third element; with the old order a mage of level 53 held three first spells at their top and every passive at level 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
classes: the measure by stage replayed on the corrected model
the measure by stage replayed on the corrected model, C30 in the place
of Calliope: 70 of 76 rows within the band
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -7941,7 +7941,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C22; C29; C34; C40</t>
+          <t>C22; C30; C34; C40</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>the user, 2026-10-09: each class measured at the stage where it is played, against several bosses of it; the class path changes at 15 and 30 (scenario.class_path)</t>
+          <t>the user, 2026-10-09: each class measured at the stage where it is played, against several bosses of it; the class path changes at 15 and 30 (scenario.class_path) | C30 in the place of C29 since 2026-10-11: the model does not play Calliope as the guide describes (docs/generated/GUIDE_CURVE.md, policy gap; Settings boss_fit_skip), and that one fight set the verdict of six roles</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the Magical Princess raises Magical Spark first
the Magical Princess raises Magical Spark first, the Kunoichi Shadow
Clone second; classes, battery and boss fit replayed

Classes 71 of 76 within the band (the Magical Princess is in; the
Kunoichi stays slow at the advanced stage), battery 65 of 85 in vanilla
and 76 of 85 on the variant.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -14065,7 +14065,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Magical Change; Sword Mastery; Magical Slash; Magic Barrier; Accelerator; Rainbow Flash; Double Attack; Magical Spark; Cover; Fireball; Ice Edge; Fire Blast</t>
+          <t>Magical Change; Sword Mastery; Magical Spark; Magical Slash; Double Attack; Magic Barrier; Accelerator; Rainbow Flash; Cover; Fireball; Ice Edge; Fire Blast</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -14075,7 +14075,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 137 (Magical Change, then her attacks; sword); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages</t>
+          <t>atwiki dt2-2 page 137 (Magical Change, then her attacks; sword); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages. Order of 2026-10-11 (choice): Magical Spark before Magical Slash and Magic Barrier. With the old order she held Magic Barrier at 10 and Magical Spark at 1, used Spark at level 1 more than any other blow, and spent her TP keeping two statuses up</t>
         </is>
       </c>
     </row>
@@ -14194,7 +14194,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Stun Sting; Sleep Sting; Dagger Mastery; Phoenix; Projectile Mastery; Dual Wield; Shadow Clone; Ninja Piledriver; Fire Scroll; Earth Scroll; Lightning Scroll; Water Scroll; Wind Scroll; Light Scroll; Shadow Sew; Barrage; Evade; Elusiveness; Adaptation</t>
+          <t>Stun Sting; Shadow Clone; Sleep Sting; Dagger Mastery; Phoenix; Projectile Mastery; Dual Wield; Ninja Piledriver; Fire Scroll; Earth Scroll; Lightning Scroll; Water Scroll; Wind Scroll; Light Scroll; Shadow Sew; Barrage; Evade; Elusiveness; Adaptation</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>atwiki dt2-2 page 142 (fast debuffer: Shadow Clone, ninja arts); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages; atwiki dt2-2 page 142: Phoenix makes a throwing weapon the main weapon, Dual Wield adds the ATK of a second weapon in the left hand (which does not count as the equipped weapon); until she is a Kunoichi she fights with a dagger and the stings of the Assassin (they need a short weapon)</t>
+          <t>atwiki dt2-2 page 142 (fast debuffer: Shadow Clone, ninja arts); GameFAQs faqs/80834 (Hentaicheg), Class Skill info pages; atwiki dt2-2 page 142: Phoenix makes a throwing weapon the main weapon, Dual Wield adds the ATK of a second weapon in the left hand (which does not count as the equipped weapon); until she is a Kunoichi she fights with a dagger and the stings of the Assassin (they need a short weapon). Order of 2026-10-11 (choice): Shadow Clone second. At level 1 it gives one dodge and she cast it again about eight times a battle</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: the superbosses fought crowned
the superbosses fought crowned, earth 100 at the fifth Aradia, and the
variant against vanilla at the preparation each fight asks for (55
bosses)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -3031,7 +3031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G207"/>
+  <dimension ref="A1:G208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9454,6 +9454,37 @@
       <c r="G207" t="inlineStr">
         <is>
           <t>atwiki dt2-2 page 326 (Plains of Light, overview): by then the party wears leather pieces and rings forged with AGI, speed and elemental resistance, seven resistance enchantments of 15 fill it, and every resistance at 100 is the premise of the dungeon; taken for every boss from there on. The enchantment slots it takes are not charged (the sheet EnchantPlan fills them apart)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>St12_0040</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>46</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>P16 Aradia (5th fight), Actim Castle</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>6</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>100</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>atwiki dt2-2 page 207: Murder License kills one member before each action of Aradia; instant death immunity (two accessories, two sealbooks) or high earth resistance is the premise of the fight</t>
         </is>
       </c>
     </row>
@@ -24684,11 +24715,11 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms) (order and boss); atwiki dt2-2 page 356 (異章, the order and the names); floor and battle matched by the name, level and HP of the enemy</t>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms) (order and boss); atwiki dt2-2 page 356 (異章, the order and the names); floor and battle matched by the name, level and HP of the enemy | Crown bonus 50 since 2026-10-12: atwiki dt2-2 page 231 (the superboss of the casino is hard even with every member crowned) and page 333 (Marduk reported as not winnable without crowns)</t>
         </is>
       </c>
     </row>
@@ -24717,11 +24748,11 @@
         <v>46</v>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms) (order and boss); atwiki dt2-2 page 356 (異章, the order and the names); floor and battle matched by the name, level and HP of the enemy</t>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms) (order and boss); atwiki dt2-2 page 356 (異章, the order and the names); floor and battle matched by the name, level and HP of the enemy | Crown bonus 50 since 2026-10-12: atwiki dt2-2 page 231 (the superboss of the casino is hard even with every member crowned) and page 333 (Marduk reported as not winnable without crowns)</t>
         </is>
       </c>
     </row>
@@ -24750,11 +24781,11 @@
         <v>46</v>
       </c>
       <c r="F92" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms) (order and boss); atwiki dt2-2 page 356 (異章, the order and the names); floor and battle matched by the name, level and HP of the enemy</t>
+          <t>GameFAQs faqs/80834 (Hentaicheg), Postgame Dungeon Superbosses(+weak forms) (order and boss); atwiki dt2-2 page 356 (異章, the order and the names); floor and battle matched by the name, level and HP of the enemy | Crown bonus 50 since 2026-10-12: atwiki dt2-2 page 231 (the superboss of the casino is hard even with every member crowned) and page 333 (Marduk reported as not winnable without crowns)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sim: every boss below its floor read
every boss below its floor read (30 readings), the comparison replayed
after the RES rows
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/sim_setup.xlsx
+++ b/mod_project/data_tables/sim_setup.xlsx
@@ -9892,7 +9892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11082,6 +11082,482 @@
       <c r="C70" t="inlineStr">
         <is>
           <t>It needs a bow or a gun; the role fights with a dagger (GameFAQs faqs/80834: she moves to a gun late).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>curve P03</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 5% at level 66 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 20, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 60%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>curve P09</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 28% at level 74 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 10, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 55%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>curve P10</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 15% at level 74 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 30, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 72%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>curve P12</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 22% at level 78 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 10, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 60%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>curve P13</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 40% at level 79 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 10, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 80%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>curve P15</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 5% at level 79 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 30, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 85%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>curve P22</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>known limit</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 84 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 12%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>curve P23</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 22% at level 84 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 20, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 70%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>curve P27</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 90 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 57%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>curve P29</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 2% at level 95 (floor of a easy boss 80%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 95%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>curve P30</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 5% at level 95 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 10, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 22%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>curve P32</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 95 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 50, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 50%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>curve P33</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>known limit</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 10%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>curve P34</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 20, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 48%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>curve P35</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 38%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>curve P36</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 5% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 32%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>curve P39</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 12% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 10, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 28%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>curve P40</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 50, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 45%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>curve P41</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>known limit</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 0%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>curve P42</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 22%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>curve P43</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 30% at level 99 (floor of a normal boss 50%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 20, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 78%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>curve P45</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 30, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 42%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>curve P46</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 8% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 10, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 45%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>curve P47</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>known limit</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 5%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>curve P48</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>preparation gap</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. With a crown bonus of 40, the stand-in of the model for that preparation (it adds to every stat and to the eight resistances), it wins 48%. Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>curve P49</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>known limit</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 0%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>curve P50</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>known limit</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 0%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>curve P51</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>known limit</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>The party of the sheets wins 0% at level 99 (floor of a hard boss 20%): it wears the gear of the guide and none of the answers a player prepares for the fight. Even with a crown bonus of 50 it wins 0%: the fight asks for an answer the policy does not play (sheet PostgameBosses, what the pages say). Measured on 2026-10-12 on the bosses below their floor (postgame_levers.py): a crown bonus of 50 alone brings 18 of 28 above it; max HP x1.5 with three pieces of "received damage DOWN" 11 of 28; the order of the Valkyrie's Cover and Parry changes nothing</t>
         </is>
       </c>
     </row>

</xml_diff>